<commit_message>
Adjusted player table to include combatant column
</commit_message>
<xml_diff>
--- a/Documentation/CRUD Table.xlsx
+++ b/Documentation/CRUD Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dyfry\workspace\2026\DAT602-Project\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBE9E0C2-379C-483F-BB87-FCF181F317D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E2A387-E485-4B3F-A3CB-45B04935B674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1075" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="87">
   <si>
     <t>Account</t>
   </si>
@@ -283,6 +283,9 @@
   </si>
   <si>
     <t>AbilityName (FK)</t>
+  </si>
+  <si>
+    <t>Combatant (FK)</t>
   </si>
 </sst>
 </file>
@@ -374,7 +377,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -382,7 +385,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1653,94 +1655,94 @@
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" t="s">
+        <v>65</v>
+      </c>
+      <c r="D19" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" t="s">
+        <v>65</v>
+      </c>
+      <c r="G19" t="s">
+        <v>65</v>
+      </c>
+      <c r="H19" t="s">
+        <v>65</v>
+      </c>
+      <c r="I19" t="s">
+        <v>65</v>
+      </c>
+      <c r="J19" t="s">
+        <v>65</v>
+      </c>
+      <c r="K19" t="s">
+        <v>65</v>
+      </c>
+      <c r="L19" t="s">
+        <v>65</v>
+      </c>
+      <c r="M19" t="s">
+        <v>65</v>
+      </c>
+      <c r="N19" t="s">
+        <v>70</v>
+      </c>
+      <c r="O19" t="s">
+        <v>65</v>
+      </c>
+      <c r="P19" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>65</v>
+      </c>
+      <c r="R19" t="s">
+        <v>69</v>
+      </c>
+      <c r="S19" t="s">
+        <v>65</v>
+      </c>
+      <c r="T19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="5"/>
-      <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="5"/>
-      <c r="L19" s="5"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
-      <c r="P19" s="5"/>
-      <c r="Q19" s="5"/>
-      <c r="R19" s="5"/>
-      <c r="S19" s="5"/>
-      <c r="T19" s="5"/>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C20" t="s">
-        <v>65</v>
-      </c>
-      <c r="D20" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" t="s">
-        <v>65</v>
-      </c>
-      <c r="F20" t="s">
-        <v>65</v>
-      </c>
-      <c r="G20" t="s">
-        <v>65</v>
-      </c>
-      <c r="H20" t="s">
-        <v>65</v>
-      </c>
-      <c r="I20" t="s">
-        <v>65</v>
-      </c>
-      <c r="J20" t="s">
-        <v>65</v>
-      </c>
-      <c r="K20" t="s">
-        <v>65</v>
-      </c>
-      <c r="L20" t="s">
-        <v>65</v>
-      </c>
-      <c r="M20" t="s">
-        <v>65</v>
-      </c>
-      <c r="N20" t="s">
-        <v>70</v>
-      </c>
-      <c r="O20" t="s">
-        <v>65</v>
-      </c>
-      <c r="P20" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q20" t="s">
-        <v>65</v>
-      </c>
-      <c r="R20" t="s">
-        <v>64</v>
-      </c>
-      <c r="S20" t="s">
-        <v>69</v>
-      </c>
-      <c r="T20" t="s">
-        <v>65</v>
-      </c>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
+      <c r="P20" s="5"/>
+      <c r="Q20" s="5"/>
+      <c r="R20" s="5"/>
+      <c r="S20" s="5"/>
+      <c r="T20" s="5"/>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
         <v>65</v>
@@ -1802,155 +1804,155 @@
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+      <c r="D22" t="s">
+        <v>65</v>
+      </c>
+      <c r="E22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" t="s">
+        <v>65</v>
+      </c>
+      <c r="G22" t="s">
+        <v>65</v>
+      </c>
+      <c r="H22" t="s">
+        <v>65</v>
+      </c>
+      <c r="I22" t="s">
+        <v>65</v>
+      </c>
+      <c r="J22" t="s">
+        <v>65</v>
+      </c>
+      <c r="K22" t="s">
+        <v>65</v>
+      </c>
+      <c r="L22" t="s">
+        <v>65</v>
+      </c>
+      <c r="M22" t="s">
+        <v>65</v>
+      </c>
+      <c r="N22" t="s">
+        <v>70</v>
+      </c>
+      <c r="O22" t="s">
+        <v>65</v>
+      </c>
+      <c r="P22" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>65</v>
+      </c>
+      <c r="R22" t="s">
+        <v>64</v>
+      </c>
+      <c r="S22" t="s">
+        <v>69</v>
+      </c>
+      <c r="T22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B22" t="s">
-        <v>65</v>
-      </c>
-      <c r="C22" t="s">
-        <v>65</v>
-      </c>
-      <c r="D22" t="s">
-        <v>65</v>
-      </c>
-      <c r="E22" t="s">
-        <v>65</v>
-      </c>
-      <c r="F22" t="s">
-        <v>65</v>
-      </c>
-      <c r="G22" t="s">
-        <v>65</v>
-      </c>
-      <c r="H22" t="s">
-        <v>65</v>
-      </c>
-      <c r="I22" t="s">
-        <v>65</v>
-      </c>
-      <c r="J22" t="s">
-        <v>65</v>
-      </c>
-      <c r="K22" t="s">
-        <v>65</v>
-      </c>
-      <c r="L22" t="s">
-        <v>65</v>
-      </c>
-      <c r="M22" t="s">
-        <v>65</v>
-      </c>
-      <c r="N22" t="s">
-        <v>70</v>
-      </c>
-      <c r="O22" t="s">
-        <v>65</v>
-      </c>
-      <c r="P22" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>65</v>
-      </c>
-      <c r="R22" t="s">
-        <v>64</v>
-      </c>
-      <c r="S22" t="s">
-        <v>69</v>
-      </c>
-      <c r="T22" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A23" s="5" t="s">
+      <c r="B23" t="s">
+        <v>65</v>
+      </c>
+      <c r="C23" t="s">
+        <v>65</v>
+      </c>
+      <c r="D23" t="s">
+        <v>65</v>
+      </c>
+      <c r="E23" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" t="s">
+        <v>65</v>
+      </c>
+      <c r="G23" t="s">
+        <v>65</v>
+      </c>
+      <c r="H23" t="s">
+        <v>65</v>
+      </c>
+      <c r="I23" t="s">
+        <v>65</v>
+      </c>
+      <c r="J23" t="s">
+        <v>65</v>
+      </c>
+      <c r="K23" t="s">
+        <v>65</v>
+      </c>
+      <c r="L23" t="s">
+        <v>65</v>
+      </c>
+      <c r="M23" t="s">
+        <v>65</v>
+      </c>
+      <c r="N23" t="s">
+        <v>70</v>
+      </c>
+      <c r="O23" t="s">
+        <v>65</v>
+      </c>
+      <c r="P23" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>65</v>
+      </c>
+      <c r="R23" t="s">
+        <v>64</v>
+      </c>
+      <c r="S23" t="s">
+        <v>69</v>
+      </c>
+      <c r="T23" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
-      <c r="P23" s="5"/>
-      <c r="Q23" s="5"/>
-      <c r="R23" s="5"/>
-      <c r="S23" s="5"/>
-      <c r="T23" s="5"/>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B24" t="s">
-        <v>65</v>
-      </c>
-      <c r="C24" t="s">
-        <v>65</v>
-      </c>
-      <c r="D24" t="s">
-        <v>65</v>
-      </c>
-      <c r="E24" t="s">
-        <v>65</v>
-      </c>
-      <c r="F24" t="s">
-        <v>65</v>
-      </c>
-      <c r="G24" t="s">
-        <v>65</v>
-      </c>
-      <c r="H24" t="s">
-        <v>65</v>
-      </c>
-      <c r="I24" t="s">
-        <v>65</v>
-      </c>
-      <c r="J24" t="s">
-        <v>65</v>
-      </c>
-      <c r="K24" t="s">
-        <v>65</v>
-      </c>
-      <c r="L24" t="s">
-        <v>65</v>
-      </c>
-      <c r="M24" t="s">
-        <v>65</v>
-      </c>
-      <c r="N24" t="s">
-        <v>70</v>
-      </c>
-      <c r="O24" t="s">
-        <v>65</v>
-      </c>
-      <c r="P24" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q24" t="s">
-        <v>65</v>
-      </c>
-      <c r="R24" t="s">
-        <v>64</v>
-      </c>
-      <c r="S24" t="s">
-        <v>65</v>
-      </c>
-      <c r="T24" t="s">
-        <v>69</v>
-      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+      <c r="N24" s="5"/>
+      <c r="O24" s="5"/>
+      <c r="P24" s="5"/>
+      <c r="Q24" s="5"/>
+      <c r="R24" s="5"/>
+      <c r="S24" s="5"/>
+      <c r="T24" s="5"/>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B25" t="s">
         <v>65</v>
@@ -2012,155 +2014,155 @@
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" t="s">
+        <v>65</v>
+      </c>
+      <c r="C26" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" t="s">
+        <v>65</v>
+      </c>
+      <c r="E26" t="s">
+        <v>65</v>
+      </c>
+      <c r="F26" t="s">
+        <v>65</v>
+      </c>
+      <c r="G26" t="s">
+        <v>65</v>
+      </c>
+      <c r="H26" t="s">
+        <v>65</v>
+      </c>
+      <c r="I26" t="s">
+        <v>65</v>
+      </c>
+      <c r="J26" t="s">
+        <v>65</v>
+      </c>
+      <c r="K26" t="s">
+        <v>65</v>
+      </c>
+      <c r="L26" t="s">
+        <v>65</v>
+      </c>
+      <c r="M26" t="s">
+        <v>65</v>
+      </c>
+      <c r="N26" t="s">
+        <v>70</v>
+      </c>
+      <c r="O26" t="s">
+        <v>65</v>
+      </c>
+      <c r="P26" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>65</v>
+      </c>
+      <c r="R26" t="s">
+        <v>64</v>
+      </c>
+      <c r="S26" t="s">
+        <v>65</v>
+      </c>
+      <c r="T26" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B26" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" t="s">
-        <v>65</v>
-      </c>
-      <c r="D26" t="s">
-        <v>65</v>
-      </c>
-      <c r="E26" t="s">
-        <v>65</v>
-      </c>
-      <c r="F26" t="s">
-        <v>65</v>
-      </c>
-      <c r="G26" t="s">
-        <v>65</v>
-      </c>
-      <c r="H26" t="s">
-        <v>65</v>
-      </c>
-      <c r="I26" t="s">
-        <v>65</v>
-      </c>
-      <c r="J26" t="s">
-        <v>65</v>
-      </c>
-      <c r="K26" t="s">
-        <v>65</v>
-      </c>
-      <c r="L26" t="s">
-        <v>65</v>
-      </c>
-      <c r="M26" t="s">
-        <v>65</v>
-      </c>
-      <c r="N26" t="s">
-        <v>70</v>
-      </c>
-      <c r="O26" t="s">
-        <v>65</v>
-      </c>
-      <c r="P26" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q26" t="s">
-        <v>65</v>
-      </c>
-      <c r="R26" t="s">
-        <v>64</v>
-      </c>
-      <c r="S26" t="s">
-        <v>65</v>
-      </c>
-      <c r="T26" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
+      <c r="B27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" t="s">
+        <v>65</v>
+      </c>
+      <c r="G27" t="s">
+        <v>65</v>
+      </c>
+      <c r="H27" t="s">
+        <v>65</v>
+      </c>
+      <c r="I27" t="s">
+        <v>65</v>
+      </c>
+      <c r="J27" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" t="s">
+        <v>65</v>
+      </c>
+      <c r="L27" t="s">
+        <v>65</v>
+      </c>
+      <c r="M27" t="s">
+        <v>65</v>
+      </c>
+      <c r="N27" t="s">
+        <v>70</v>
+      </c>
+      <c r="O27" t="s">
+        <v>65</v>
+      </c>
+      <c r="P27" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q27" t="s">
+        <v>65</v>
+      </c>
+      <c r="R27" t="s">
+        <v>64</v>
+      </c>
+      <c r="S27" t="s">
+        <v>65</v>
+      </c>
+      <c r="T27" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-      <c r="O27" s="5"/>
-      <c r="P27" s="5"/>
-      <c r="Q27" s="5"/>
-      <c r="R27" s="5"/>
-      <c r="S27" s="5"/>
-      <c r="T27" s="5"/>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B28" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" t="s">
-        <v>65</v>
-      </c>
-      <c r="D28" t="s">
-        <v>65</v>
-      </c>
-      <c r="E28" t="s">
-        <v>65</v>
-      </c>
-      <c r="F28" t="s">
-        <v>65</v>
-      </c>
-      <c r="G28" t="s">
-        <v>65</v>
-      </c>
-      <c r="H28" t="s">
-        <v>69</v>
-      </c>
-      <c r="I28" t="s">
-        <v>65</v>
-      </c>
-      <c r="J28" t="s">
-        <v>65</v>
-      </c>
-      <c r="K28" t="s">
-        <v>65</v>
-      </c>
-      <c r="L28" t="s">
-        <v>69</v>
-      </c>
-      <c r="M28" t="s">
-        <v>64</v>
-      </c>
-      <c r="N28" t="s">
-        <v>70</v>
-      </c>
-      <c r="O28" t="s">
-        <v>65</v>
-      </c>
-      <c r="P28" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>65</v>
-      </c>
-      <c r="R28" t="s">
-        <v>64</v>
-      </c>
-      <c r="S28" t="s">
-        <v>65</v>
-      </c>
-      <c r="T28" t="s">
-        <v>65</v>
-      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+      <c r="O28" s="5"/>
+      <c r="P28" s="5"/>
+      <c r="Q28" s="5"/>
+      <c r="R28" s="5"/>
+      <c r="S28" s="5"/>
+      <c r="T28" s="5"/>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
         <v>65</v>
@@ -2222,155 +2224,155 @@
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>65</v>
+      </c>
+      <c r="D30" t="s">
+        <v>65</v>
+      </c>
+      <c r="E30" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" t="s">
+        <v>65</v>
+      </c>
+      <c r="G30" t="s">
+        <v>65</v>
+      </c>
+      <c r="H30" t="s">
+        <v>69</v>
+      </c>
+      <c r="I30" t="s">
+        <v>65</v>
+      </c>
+      <c r="J30" t="s">
+        <v>65</v>
+      </c>
+      <c r="K30" t="s">
+        <v>65</v>
+      </c>
+      <c r="L30" t="s">
+        <v>69</v>
+      </c>
+      <c r="M30" t="s">
+        <v>64</v>
+      </c>
+      <c r="N30" t="s">
+        <v>70</v>
+      </c>
+      <c r="O30" t="s">
+        <v>65</v>
+      </c>
+      <c r="P30" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>65</v>
+      </c>
+      <c r="R30" t="s">
+        <v>64</v>
+      </c>
+      <c r="S30" t="s">
+        <v>65</v>
+      </c>
+      <c r="T30" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C30" t="s">
-        <v>65</v>
-      </c>
-      <c r="D30" t="s">
-        <v>65</v>
-      </c>
-      <c r="E30" t="s">
-        <v>65</v>
-      </c>
-      <c r="F30" t="s">
-        <v>65</v>
-      </c>
-      <c r="G30" t="s">
-        <v>65</v>
-      </c>
-      <c r="H30" t="s">
-        <v>69</v>
-      </c>
-      <c r="I30" t="s">
-        <v>65</v>
-      </c>
-      <c r="J30" t="s">
-        <v>65</v>
-      </c>
-      <c r="K30" t="s">
-        <v>65</v>
-      </c>
-      <c r="L30" t="s">
-        <v>69</v>
-      </c>
-      <c r="M30" t="s">
-        <v>64</v>
-      </c>
-      <c r="N30" t="s">
-        <v>70</v>
-      </c>
-      <c r="O30" t="s">
-        <v>65</v>
-      </c>
-      <c r="P30" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q30" t="s">
-        <v>65</v>
-      </c>
-      <c r="R30" t="s">
-        <v>64</v>
-      </c>
-      <c r="S30" t="s">
-        <v>65</v>
-      </c>
-      <c r="T30" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="B31" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" t="s">
+        <v>65</v>
+      </c>
+      <c r="F31" t="s">
+        <v>65</v>
+      </c>
+      <c r="G31" t="s">
+        <v>65</v>
+      </c>
+      <c r="H31" t="s">
+        <v>69</v>
+      </c>
+      <c r="I31" t="s">
+        <v>65</v>
+      </c>
+      <c r="J31" t="s">
+        <v>65</v>
+      </c>
+      <c r="K31" t="s">
+        <v>65</v>
+      </c>
+      <c r="L31" t="s">
+        <v>69</v>
+      </c>
+      <c r="M31" t="s">
+        <v>64</v>
+      </c>
+      <c r="N31" t="s">
+        <v>70</v>
+      </c>
+      <c r="O31" t="s">
+        <v>65</v>
+      </c>
+      <c r="P31" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>65</v>
+      </c>
+      <c r="R31" t="s">
+        <v>64</v>
+      </c>
+      <c r="S31" t="s">
+        <v>65</v>
+      </c>
+      <c r="T31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="5"/>
-      <c r="C31" s="5"/>
-      <c r="D31" s="5"/>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5"/>
-      <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-      <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
-      <c r="K31" s="5"/>
-      <c r="L31" s="5"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="5"/>
-      <c r="O31" s="5"/>
-      <c r="P31" s="5"/>
-      <c r="Q31" s="5"/>
-      <c r="R31" s="5"/>
-      <c r="S31" s="5"/>
-      <c r="T31" s="5"/>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A32" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B32" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" t="s">
-        <v>65</v>
-      </c>
-      <c r="E32" t="s">
-        <v>65</v>
-      </c>
-      <c r="F32" t="s">
-        <v>64</v>
-      </c>
-      <c r="G32" t="s">
-        <v>64</v>
-      </c>
-      <c r="H32" t="s">
-        <v>64</v>
-      </c>
-      <c r="I32" t="s">
-        <v>65</v>
-      </c>
-      <c r="J32" t="s">
-        <v>64</v>
-      </c>
-      <c r="K32" t="s">
-        <v>65</v>
-      </c>
-      <c r="L32" t="s">
-        <v>64</v>
-      </c>
-      <c r="M32" t="s">
-        <v>64</v>
-      </c>
-      <c r="N32" t="s">
-        <v>70</v>
-      </c>
-      <c r="O32" t="s">
-        <v>65</v>
-      </c>
-      <c r="P32" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q32" t="s">
-        <v>65</v>
-      </c>
-      <c r="R32" t="s">
-        <v>64</v>
-      </c>
-      <c r="S32" t="s">
-        <v>65</v>
-      </c>
-      <c r="T32" t="s">
-        <v>69</v>
-      </c>
+      <c r="B32" s="5"/>
+      <c r="C32" s="5"/>
+      <c r="D32" s="5"/>
+      <c r="E32" s="5"/>
+      <c r="F32" s="5"/>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+      <c r="N32" s="5"/>
+      <c r="O32" s="5"/>
+      <c r="P32" s="5"/>
+      <c r="Q32" s="5"/>
+      <c r="R32" s="5"/>
+      <c r="S32" s="5"/>
+      <c r="T32" s="5"/>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B33" t="s">
         <v>65</v>
@@ -2388,25 +2390,25 @@
         <v>64</v>
       </c>
       <c r="G33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I33" t="s">
         <v>65</v>
       </c>
       <c r="J33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K33" t="s">
         <v>65</v>
       </c>
       <c r="L33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M33" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N33" t="s">
         <v>70</v>
@@ -2432,7 +2434,7 @@
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B34" t="s">
         <v>65</v>
@@ -2494,155 +2496,155 @@
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" t="s">
+        <v>65</v>
+      </c>
+      <c r="D35" t="s">
+        <v>65</v>
+      </c>
+      <c r="E35" t="s">
+        <v>65</v>
+      </c>
+      <c r="F35" t="s">
+        <v>64</v>
+      </c>
+      <c r="G35" t="s">
+        <v>65</v>
+      </c>
+      <c r="H35" t="s">
+        <v>65</v>
+      </c>
+      <c r="I35" t="s">
+        <v>65</v>
+      </c>
+      <c r="J35" t="s">
+        <v>65</v>
+      </c>
+      <c r="K35" t="s">
+        <v>65</v>
+      </c>
+      <c r="L35" t="s">
+        <v>65</v>
+      </c>
+      <c r="M35" t="s">
+        <v>65</v>
+      </c>
+      <c r="N35" t="s">
+        <v>70</v>
+      </c>
+      <c r="O35" t="s">
+        <v>65</v>
+      </c>
+      <c r="P35" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>65</v>
+      </c>
+      <c r="R35" t="s">
+        <v>64</v>
+      </c>
+      <c r="S35" t="s">
+        <v>65</v>
+      </c>
+      <c r="T35" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B35" t="s">
-        <v>65</v>
-      </c>
-      <c r="C35" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" t="s">
-        <v>65</v>
-      </c>
-      <c r="E35" t="s">
-        <v>65</v>
-      </c>
-      <c r="F35" t="s">
-        <v>64</v>
-      </c>
-      <c r="G35" t="s">
-        <v>65</v>
-      </c>
-      <c r="H35" t="s">
-        <v>65</v>
-      </c>
-      <c r="I35" t="s">
-        <v>65</v>
-      </c>
-      <c r="J35" t="s">
-        <v>65</v>
-      </c>
-      <c r="K35" t="s">
-        <v>65</v>
-      </c>
-      <c r="L35" t="s">
-        <v>65</v>
-      </c>
-      <c r="M35" t="s">
-        <v>65</v>
-      </c>
-      <c r="N35" t="s">
-        <v>70</v>
-      </c>
-      <c r="O35" t="s">
-        <v>65</v>
-      </c>
-      <c r="P35" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q35" t="s">
-        <v>65</v>
-      </c>
-      <c r="R35" t="s">
-        <v>64</v>
-      </c>
-      <c r="S35" t="s">
-        <v>65</v>
-      </c>
-      <c r="T35" t="s">
+      <c r="B36" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36" t="s">
+        <v>65</v>
+      </c>
+      <c r="F36" t="s">
+        <v>64</v>
+      </c>
+      <c r="G36" t="s">
+        <v>65</v>
+      </c>
+      <c r="H36" t="s">
+        <v>65</v>
+      </c>
+      <c r="I36" t="s">
+        <v>65</v>
+      </c>
+      <c r="J36" t="s">
+        <v>65</v>
+      </c>
+      <c r="K36" t="s">
+        <v>65</v>
+      </c>
+      <c r="L36" t="s">
+        <v>65</v>
+      </c>
+      <c r="M36" t="s">
+        <v>65</v>
+      </c>
+      <c r="N36" t="s">
+        <v>70</v>
+      </c>
+      <c r="O36" t="s">
+        <v>65</v>
+      </c>
+      <c r="P36" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>65</v>
+      </c>
+      <c r="R36" t="s">
+        <v>64</v>
+      </c>
+      <c r="S36" t="s">
+        <v>65</v>
+      </c>
+      <c r="T36" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A36" s="5" t="s">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A37" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B36" s="5"/>
-      <c r="C36" s="5"/>
-      <c r="D36" s="5"/>
-      <c r="E36" s="5"/>
-      <c r="F36" s="5"/>
-      <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-      <c r="K36" s="5"/>
-      <c r="L36" s="5"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="5"/>
-      <c r="O36" s="5"/>
-      <c r="P36" s="5"/>
-      <c r="Q36" s="5"/>
-      <c r="R36" s="5"/>
-      <c r="S36" s="5"/>
-      <c r="T36" s="5"/>
-    </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A37" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B37" t="s">
-        <v>65</v>
-      </c>
-      <c r="C37" t="s">
-        <v>65</v>
-      </c>
-      <c r="D37" t="s">
-        <v>65</v>
-      </c>
-      <c r="E37" t="s">
-        <v>65</v>
-      </c>
-      <c r="F37" t="s">
-        <v>65</v>
-      </c>
-      <c r="G37" t="s">
-        <v>69</v>
-      </c>
-      <c r="H37" t="s">
-        <v>64</v>
-      </c>
-      <c r="I37" t="s">
-        <v>64</v>
-      </c>
-      <c r="J37" t="s">
-        <v>69</v>
-      </c>
-      <c r="K37" t="s">
-        <v>65</v>
-      </c>
-      <c r="L37" t="s">
-        <v>65</v>
-      </c>
-      <c r="M37" t="s">
-        <v>68</v>
-      </c>
-      <c r="N37" t="s">
-        <v>70</v>
-      </c>
-      <c r="O37" t="s">
-        <v>65</v>
-      </c>
-      <c r="P37" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>65</v>
-      </c>
-      <c r="R37" t="s">
-        <v>64</v>
-      </c>
-      <c r="S37" t="s">
-        <v>65</v>
-      </c>
-      <c r="T37" t="s">
-        <v>65</v>
-      </c>
+      <c r="B37" s="5"/>
+      <c r="C37" s="5"/>
+      <c r="D37" s="5"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="5"/>
+      <c r="H37" s="5"/>
+      <c r="I37" s="5"/>
+      <c r="J37" s="5"/>
+      <c r="K37" s="5"/>
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+      <c r="N37" s="5"/>
+      <c r="O37" s="5"/>
+      <c r="P37" s="5"/>
+      <c r="Q37" s="5"/>
+      <c r="R37" s="5"/>
+      <c r="S37" s="5"/>
+      <c r="T37" s="5"/>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="B38" t="s">
         <v>65</v>
@@ -2704,7 +2706,7 @@
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s">
         <v>65</v>
@@ -2766,7 +2768,7 @@
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B40" t="s">
         <v>65</v>
@@ -2784,16 +2786,16 @@
         <v>65</v>
       </c>
       <c r="G40" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H40" t="s">
         <v>64</v>
       </c>
       <c r="I40" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="J40" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="K40" t="s">
         <v>65</v>
@@ -2827,94 +2829,94 @@
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B41" t="s">
+        <v>65</v>
+      </c>
+      <c r="C41" t="s">
+        <v>65</v>
+      </c>
+      <c r="D41" t="s">
+        <v>65</v>
+      </c>
+      <c r="E41" t="s">
+        <v>65</v>
+      </c>
+      <c r="F41" t="s">
+        <v>65</v>
+      </c>
+      <c r="G41" t="s">
+        <v>65</v>
+      </c>
+      <c r="H41" t="s">
+        <v>64</v>
+      </c>
+      <c r="I41" t="s">
+        <v>69</v>
+      </c>
+      <c r="J41" t="s">
+        <v>65</v>
+      </c>
+      <c r="K41" t="s">
+        <v>65</v>
+      </c>
+      <c r="L41" t="s">
+        <v>65</v>
+      </c>
+      <c r="M41" t="s">
+        <v>68</v>
+      </c>
+      <c r="N41" t="s">
+        <v>70</v>
+      </c>
+      <c r="O41" t="s">
+        <v>65</v>
+      </c>
+      <c r="P41" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q41" t="s">
+        <v>65</v>
+      </c>
+      <c r="R41" t="s">
+        <v>64</v>
+      </c>
+      <c r="S41" t="s">
+        <v>65</v>
+      </c>
+      <c r="T41" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B41" s="5"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="5"/>
-      <c r="E41" s="5"/>
-      <c r="F41" s="5"/>
-      <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-      <c r="I41" s="5"/>
-      <c r="J41" s="5"/>
-      <c r="K41" s="5"/>
-      <c r="L41" s="5"/>
-      <c r="M41" s="5"/>
-      <c r="N41" s="5"/>
-      <c r="O41" s="5"/>
-      <c r="P41" s="5"/>
-      <c r="Q41" s="5"/>
-      <c r="R41" s="5"/>
-      <c r="S41" s="5"/>
-      <c r="T41" s="5"/>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B42" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" t="s">
-        <v>65</v>
-      </c>
-      <c r="D42" t="s">
-        <v>65</v>
-      </c>
-      <c r="E42" t="s">
-        <v>65</v>
-      </c>
-      <c r="F42" t="s">
-        <v>65</v>
-      </c>
-      <c r="G42" t="s">
-        <v>68</v>
-      </c>
-      <c r="H42" t="s">
-        <v>65</v>
-      </c>
-      <c r="I42" t="s">
-        <v>64</v>
-      </c>
-      <c r="J42" t="s">
-        <v>64</v>
-      </c>
-      <c r="K42" t="s">
-        <v>65</v>
-      </c>
-      <c r="L42" t="s">
-        <v>65</v>
-      </c>
-      <c r="M42" t="s">
-        <v>65</v>
-      </c>
-      <c r="N42" t="s">
-        <v>65</v>
-      </c>
-      <c r="O42" t="s">
-        <v>65</v>
-      </c>
-      <c r="P42" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q42" t="s">
-        <v>65</v>
-      </c>
-      <c r="R42" t="s">
-        <v>64</v>
-      </c>
-      <c r="S42" t="s">
-        <v>65</v>
-      </c>
-      <c r="T42" t="s">
-        <v>65</v>
-      </c>
+      <c r="B42" s="5"/>
+      <c r="C42" s="5"/>
+      <c r="D42" s="5"/>
+      <c r="E42" s="5"/>
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="5"/>
+      <c r="L42" s="5"/>
+      <c r="M42" s="5"/>
+      <c r="N42" s="5"/>
+      <c r="O42" s="5"/>
+      <c r="P42" s="5"/>
+      <c r="Q42" s="5"/>
+      <c r="R42" s="5"/>
+      <c r="S42" s="5"/>
+      <c r="T42" s="5"/>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="B43" t="s">
         <v>65</v>
@@ -2976,7 +2978,7 @@
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B44" t="s">
         <v>65</v>
@@ -3038,7 +3040,7 @@
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45" t="s">
         <v>65</v>
@@ -3100,7 +3102,7 @@
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B46" t="s">
         <v>65</v>
@@ -3162,7 +3164,7 @@
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B47" t="s">
         <v>65</v>
@@ -3224,7 +3226,7 @@
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B48" t="s">
         <v>65</v>
@@ -3286,7 +3288,7 @@
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B49" t="s">
         <v>65</v>
@@ -3347,94 +3349,94 @@
       </c>
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B50" t="s">
+        <v>65</v>
+      </c>
+      <c r="C50" t="s">
+        <v>65</v>
+      </c>
+      <c r="D50" t="s">
+        <v>65</v>
+      </c>
+      <c r="E50" t="s">
+        <v>65</v>
+      </c>
+      <c r="F50" t="s">
+        <v>65</v>
+      </c>
+      <c r="G50" t="s">
+        <v>68</v>
+      </c>
+      <c r="H50" t="s">
+        <v>65</v>
+      </c>
+      <c r="I50" t="s">
+        <v>64</v>
+      </c>
+      <c r="J50" t="s">
+        <v>64</v>
+      </c>
+      <c r="K50" t="s">
+        <v>65</v>
+      </c>
+      <c r="L50" t="s">
+        <v>65</v>
+      </c>
+      <c r="M50" t="s">
+        <v>65</v>
+      </c>
+      <c r="N50" t="s">
+        <v>65</v>
+      </c>
+      <c r="O50" t="s">
+        <v>65</v>
+      </c>
+      <c r="P50" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>65</v>
+      </c>
+      <c r="R50" t="s">
+        <v>64</v>
+      </c>
+      <c r="S50" t="s">
+        <v>65</v>
+      </c>
+      <c r="T50" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B50" s="5"/>
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="5"/>
-      <c r="J50" s="5"/>
-      <c r="K50" s="5"/>
-      <c r="L50" s="5"/>
-      <c r="M50" s="5"/>
-      <c r="N50" s="5"/>
-      <c r="O50" s="5"/>
-      <c r="P50" s="5"/>
-      <c r="Q50" s="5"/>
-      <c r="R50" s="5"/>
-      <c r="S50" s="5"/>
-      <c r="T50" s="5"/>
-    </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A51" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B51" t="s">
-        <v>65</v>
-      </c>
-      <c r="C51" t="s">
-        <v>65</v>
-      </c>
-      <c r="D51" t="s">
-        <v>65</v>
-      </c>
-      <c r="E51" t="s">
-        <v>65</v>
-      </c>
-      <c r="F51" t="s">
-        <v>65</v>
-      </c>
-      <c r="G51" t="s">
-        <v>65</v>
-      </c>
-      <c r="H51" t="s">
-        <v>65</v>
-      </c>
-      <c r="I51" t="s">
-        <v>69</v>
-      </c>
-      <c r="J51" t="s">
-        <v>64</v>
-      </c>
-      <c r="K51" t="s">
-        <v>65</v>
-      </c>
-      <c r="L51" t="s">
-        <v>64</v>
-      </c>
-      <c r="M51" t="s">
-        <v>65</v>
-      </c>
-      <c r="N51" t="s">
-        <v>70</v>
-      </c>
-      <c r="O51" t="s">
-        <v>65</v>
-      </c>
-      <c r="P51" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q51" t="s">
-        <v>65</v>
-      </c>
-      <c r="R51" t="s">
-        <v>64</v>
-      </c>
-      <c r="S51" t="s">
-        <v>65</v>
-      </c>
-      <c r="T51" t="s">
-        <v>65</v>
-      </c>
+      <c r="B51" s="5"/>
+      <c r="C51" s="5"/>
+      <c r="D51" s="5"/>
+      <c r="E51" s="5"/>
+      <c r="F51" s="5"/>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+      <c r="N51" s="5"/>
+      <c r="O51" s="5"/>
+      <c r="P51" s="5"/>
+      <c r="Q51" s="5"/>
+      <c r="R51" s="5"/>
+      <c r="S51" s="5"/>
+      <c r="T51" s="5"/>
     </row>
     <row r="52" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="B52" t="s">
         <v>65</v>
@@ -3464,7 +3466,7 @@
         <v>64</v>
       </c>
       <c r="K52" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L52" t="s">
         <v>64</v>
@@ -3496,7 +3498,7 @@
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="B53" t="s">
         <v>65</v>
@@ -3558,155 +3560,155 @@
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B54" t="s">
+        <v>65</v>
+      </c>
+      <c r="C54" t="s">
+        <v>65</v>
+      </c>
+      <c r="D54" t="s">
+        <v>65</v>
+      </c>
+      <c r="E54" t="s">
+        <v>65</v>
+      </c>
+      <c r="F54" t="s">
+        <v>65</v>
+      </c>
+      <c r="G54" t="s">
+        <v>65</v>
+      </c>
+      <c r="H54" t="s">
+        <v>65</v>
+      </c>
+      <c r="I54" t="s">
+        <v>69</v>
+      </c>
+      <c r="J54" t="s">
+        <v>64</v>
+      </c>
+      <c r="K54" t="s">
+        <v>64</v>
+      </c>
+      <c r="L54" t="s">
+        <v>64</v>
+      </c>
+      <c r="M54" t="s">
+        <v>65</v>
+      </c>
+      <c r="N54" t="s">
+        <v>70</v>
+      </c>
+      <c r="O54" t="s">
+        <v>65</v>
+      </c>
+      <c r="P54" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q54" t="s">
+        <v>65</v>
+      </c>
+      <c r="R54" t="s">
+        <v>64</v>
+      </c>
+      <c r="S54" t="s">
+        <v>65</v>
+      </c>
+      <c r="T54" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A55" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B54" t="s">
-        <v>65</v>
-      </c>
-      <c r="C54" t="s">
-        <v>65</v>
-      </c>
-      <c r="D54" t="s">
-        <v>65</v>
-      </c>
-      <c r="E54" t="s">
-        <v>65</v>
-      </c>
-      <c r="F54" t="s">
-        <v>65</v>
-      </c>
-      <c r="G54" t="s">
-        <v>65</v>
-      </c>
-      <c r="H54" t="s">
-        <v>65</v>
-      </c>
-      <c r="I54" t="s">
-        <v>69</v>
-      </c>
-      <c r="J54" t="s">
+      <c r="B55" t="s">
+        <v>65</v>
+      </c>
+      <c r="C55" t="s">
+        <v>65</v>
+      </c>
+      <c r="D55" t="s">
+        <v>65</v>
+      </c>
+      <c r="E55" t="s">
+        <v>65</v>
+      </c>
+      <c r="F55" t="s">
+        <v>65</v>
+      </c>
+      <c r="G55" t="s">
+        <v>65</v>
+      </c>
+      <c r="H55" t="s">
+        <v>65</v>
+      </c>
+      <c r="I55" t="s">
+        <v>69</v>
+      </c>
+      <c r="J55" t="s">
         <v>66</v>
       </c>
-      <c r="K54" t="s">
-        <v>64</v>
-      </c>
-      <c r="L54" t="s">
+      <c r="K55" t="s">
+        <v>64</v>
+      </c>
+      <c r="L55" t="s">
         <v>66</v>
       </c>
-      <c r="M54" t="s">
-        <v>65</v>
-      </c>
-      <c r="N54" t="s">
-        <v>70</v>
-      </c>
-      <c r="O54" t="s">
-        <v>65</v>
-      </c>
-      <c r="P54" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q54" t="s">
-        <v>65</v>
-      </c>
-      <c r="R54" t="s">
-        <v>64</v>
-      </c>
-      <c r="S54" t="s">
-        <v>65</v>
-      </c>
-      <c r="T54" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A55" s="5" t="s">
+      <c r="M55" t="s">
+        <v>65</v>
+      </c>
+      <c r="N55" t="s">
+        <v>70</v>
+      </c>
+      <c r="O55" t="s">
+        <v>65</v>
+      </c>
+      <c r="P55" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>65</v>
+      </c>
+      <c r="R55" t="s">
+        <v>64</v>
+      </c>
+      <c r="S55" t="s">
+        <v>65</v>
+      </c>
+      <c r="T55" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B55" s="5"/>
-      <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-      <c r="J55" s="5"/>
-      <c r="K55" s="5"/>
-      <c r="L55" s="5"/>
-      <c r="M55" s="5"/>
-      <c r="N55" s="5"/>
-      <c r="O55" s="5"/>
-      <c r="P55" s="5"/>
-      <c r="Q55" s="5"/>
-      <c r="R55" s="5"/>
-      <c r="S55" s="5"/>
-      <c r="T55" s="5"/>
-    </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A56" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B56" t="s">
-        <v>65</v>
-      </c>
-      <c r="C56" t="s">
-        <v>65</v>
-      </c>
-      <c r="D56" t="s">
-        <v>65</v>
-      </c>
-      <c r="E56" t="s">
-        <v>65</v>
-      </c>
-      <c r="F56" t="s">
-        <v>65</v>
-      </c>
-      <c r="G56" t="s">
-        <v>69</v>
-      </c>
-      <c r="H56" t="s">
-        <v>65</v>
-      </c>
-      <c r="I56" t="s">
-        <v>64</v>
-      </c>
-      <c r="J56" t="s">
-        <v>65</v>
-      </c>
-      <c r="K56" t="s">
-        <v>65</v>
-      </c>
-      <c r="L56" t="s">
-        <v>65</v>
-      </c>
-      <c r="M56" t="s">
-        <v>65</v>
-      </c>
-      <c r="N56" t="s">
-        <v>65</v>
-      </c>
-      <c r="O56" t="s">
-        <v>65</v>
-      </c>
-      <c r="P56" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q56" t="s">
-        <v>65</v>
-      </c>
-      <c r="R56" t="s">
-        <v>64</v>
-      </c>
-      <c r="S56" t="s">
-        <v>65</v>
-      </c>
-      <c r="T56" t="s">
-        <v>65</v>
-      </c>
+      <c r="B56" s="5"/>
+      <c r="C56" s="5"/>
+      <c r="D56" s="5"/>
+      <c r="E56" s="5"/>
+      <c r="F56" s="5"/>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="K56" s="5"/>
+      <c r="L56" s="5"/>
+      <c r="M56" s="5"/>
+      <c r="N56" s="5"/>
+      <c r="O56" s="5"/>
+      <c r="P56" s="5"/>
+      <c r="Q56" s="5"/>
+      <c r="R56" s="5"/>
+      <c r="S56" s="5"/>
+      <c r="T56" s="5"/>
     </row>
     <row r="57" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B57" t="s">
         <v>65</v>
@@ -3768,303 +3770,303 @@
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" t="s">
+        <v>65</v>
+      </c>
+      <c r="C58" t="s">
+        <v>65</v>
+      </c>
+      <c r="D58" t="s">
+        <v>65</v>
+      </c>
+      <c r="E58" t="s">
+        <v>65</v>
+      </c>
+      <c r="F58" t="s">
+        <v>65</v>
+      </c>
+      <c r="G58" t="s">
+        <v>69</v>
+      </c>
+      <c r="H58" t="s">
+        <v>65</v>
+      </c>
+      <c r="I58" t="s">
+        <v>64</v>
+      </c>
+      <c r="J58" t="s">
+        <v>65</v>
+      </c>
+      <c r="K58" t="s">
+        <v>65</v>
+      </c>
+      <c r="L58" t="s">
+        <v>65</v>
+      </c>
+      <c r="M58" t="s">
+        <v>65</v>
+      </c>
+      <c r="N58" t="s">
+        <v>65</v>
+      </c>
+      <c r="O58" t="s">
+        <v>65</v>
+      </c>
+      <c r="P58" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>65</v>
+      </c>
+      <c r="R58" t="s">
+        <v>64</v>
+      </c>
+      <c r="S58" t="s">
+        <v>65</v>
+      </c>
+      <c r="T58" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A59" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B58" t="s">
-        <v>65</v>
-      </c>
-      <c r="C58" t="s">
-        <v>65</v>
-      </c>
-      <c r="D58" t="s">
-        <v>65</v>
-      </c>
-      <c r="E58" t="s">
-        <v>65</v>
-      </c>
-      <c r="F58" t="s">
-        <v>65</v>
-      </c>
-      <c r="G58" t="s">
-        <v>69</v>
-      </c>
-      <c r="H58" t="s">
-        <v>65</v>
-      </c>
-      <c r="I58" t="s">
-        <v>64</v>
-      </c>
-      <c r="J58" t="s">
-        <v>65</v>
-      </c>
-      <c r="K58" t="s">
-        <v>65</v>
-      </c>
-      <c r="L58" t="s">
-        <v>65</v>
-      </c>
-      <c r="M58" t="s">
-        <v>65</v>
-      </c>
-      <c r="N58" t="s">
-        <v>65</v>
-      </c>
-      <c r="O58" t="s">
-        <v>65</v>
-      </c>
-      <c r="P58" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q58" t="s">
-        <v>65</v>
-      </c>
-      <c r="R58" t="s">
-        <v>64</v>
-      </c>
-      <c r="S58" t="s">
-        <v>65</v>
-      </c>
-      <c r="T58" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A59" s="5" t="s">
+      <c r="B59" t="s">
+        <v>65</v>
+      </c>
+      <c r="C59" t="s">
+        <v>65</v>
+      </c>
+      <c r="D59" t="s">
+        <v>65</v>
+      </c>
+      <c r="E59" t="s">
+        <v>65</v>
+      </c>
+      <c r="F59" t="s">
+        <v>65</v>
+      </c>
+      <c r="G59" t="s">
+        <v>69</v>
+      </c>
+      <c r="H59" t="s">
+        <v>65</v>
+      </c>
+      <c r="I59" t="s">
+        <v>64</v>
+      </c>
+      <c r="J59" t="s">
+        <v>65</v>
+      </c>
+      <c r="K59" t="s">
+        <v>65</v>
+      </c>
+      <c r="L59" t="s">
+        <v>65</v>
+      </c>
+      <c r="M59" t="s">
+        <v>65</v>
+      </c>
+      <c r="N59" t="s">
+        <v>65</v>
+      </c>
+      <c r="O59" t="s">
+        <v>65</v>
+      </c>
+      <c r="P59" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q59" t="s">
+        <v>65</v>
+      </c>
+      <c r="R59" t="s">
+        <v>64</v>
+      </c>
+      <c r="S59" t="s">
+        <v>65</v>
+      </c>
+      <c r="T59" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B59" s="5"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
-      <c r="E59" s="5"/>
-      <c r="F59" s="5"/>
-      <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
-      <c r="K59" s="5"/>
-      <c r="L59" s="5"/>
-      <c r="M59" s="5"/>
-      <c r="N59" s="5"/>
-      <c r="O59" s="5"/>
-      <c r="P59" s="5"/>
-      <c r="Q59" s="5"/>
-      <c r="R59" s="5"/>
-      <c r="S59" s="5"/>
-      <c r="T59" s="5"/>
-    </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A60" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B60" t="s">
-        <v>65</v>
-      </c>
-      <c r="C60" t="s">
-        <v>65</v>
-      </c>
-      <c r="D60" t="s">
-        <v>65</v>
-      </c>
-      <c r="E60" t="s">
-        <v>65</v>
-      </c>
-      <c r="F60" t="s">
-        <v>65</v>
-      </c>
-      <c r="G60" t="s">
-        <v>69</v>
-      </c>
-      <c r="H60" t="s">
-        <v>65</v>
-      </c>
-      <c r="I60" t="s">
-        <v>64</v>
-      </c>
-      <c r="J60" t="s">
-        <v>65</v>
-      </c>
-      <c r="K60" t="s">
-        <v>65</v>
-      </c>
-      <c r="L60" t="s">
-        <v>65</v>
-      </c>
-      <c r="M60" t="s">
-        <v>65</v>
-      </c>
-      <c r="N60" t="s">
-        <v>65</v>
-      </c>
-      <c r="O60" t="s">
-        <v>65</v>
-      </c>
-      <c r="P60" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q60" t="s">
-        <v>65</v>
-      </c>
-      <c r="R60" t="s">
-        <v>64</v>
-      </c>
-      <c r="S60" t="s">
-        <v>65</v>
-      </c>
-      <c r="T60" t="s">
-        <v>65</v>
-      </c>
+      <c r="B60" s="5"/>
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="5"/>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="5"/>
+      <c r="K60" s="5"/>
+      <c r="L60" s="5"/>
+      <c r="M60" s="5"/>
+      <c r="N60" s="5"/>
+      <c r="O60" s="5"/>
+      <c r="P60" s="5"/>
+      <c r="Q60" s="5"/>
+      <c r="R60" s="5"/>
+      <c r="S60" s="5"/>
+      <c r="T60" s="5"/>
     </row>
     <row r="61" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B61" t="s">
+        <v>65</v>
+      </c>
+      <c r="C61" t="s">
+        <v>65</v>
+      </c>
+      <c r="D61" t="s">
+        <v>65</v>
+      </c>
+      <c r="E61" t="s">
+        <v>65</v>
+      </c>
+      <c r="F61" t="s">
+        <v>65</v>
+      </c>
+      <c r="G61" t="s">
+        <v>69</v>
+      </c>
+      <c r="H61" t="s">
+        <v>65</v>
+      </c>
+      <c r="I61" t="s">
+        <v>64</v>
+      </c>
+      <c r="J61" t="s">
+        <v>65</v>
+      </c>
+      <c r="K61" t="s">
+        <v>65</v>
+      </c>
+      <c r="L61" t="s">
+        <v>65</v>
+      </c>
+      <c r="M61" t="s">
+        <v>65</v>
+      </c>
+      <c r="N61" t="s">
+        <v>65</v>
+      </c>
+      <c r="O61" t="s">
+        <v>65</v>
+      </c>
+      <c r="P61" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q61" t="s">
+        <v>65</v>
+      </c>
+      <c r="R61" t="s">
+        <v>64</v>
+      </c>
+      <c r="S61" t="s">
+        <v>65</v>
+      </c>
+      <c r="T61" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A62" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B61" t="s">
-        <v>65</v>
-      </c>
-      <c r="C61" t="s">
-        <v>65</v>
-      </c>
-      <c r="D61" t="s">
-        <v>65</v>
-      </c>
-      <c r="E61" t="s">
-        <v>65</v>
-      </c>
-      <c r="F61" t="s">
-        <v>65</v>
-      </c>
-      <c r="G61" t="s">
-        <v>69</v>
-      </c>
-      <c r="H61" t="s">
-        <v>65</v>
-      </c>
-      <c r="I61" t="s">
-        <v>64</v>
-      </c>
-      <c r="J61" t="s">
-        <v>65</v>
-      </c>
-      <c r="K61" t="s">
-        <v>65</v>
-      </c>
-      <c r="L61" t="s">
-        <v>65</v>
-      </c>
-      <c r="M61" t="s">
-        <v>65</v>
-      </c>
-      <c r="N61" t="s">
-        <v>65</v>
-      </c>
-      <c r="O61" t="s">
-        <v>65</v>
-      </c>
-      <c r="P61" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q61" t="s">
-        <v>65</v>
-      </c>
-      <c r="R61" t="s">
-        <v>64</v>
-      </c>
-      <c r="S61" t="s">
-        <v>65</v>
-      </c>
-      <c r="T61" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A62" s="5" t="s">
+      <c r="B62" t="s">
+        <v>65</v>
+      </c>
+      <c r="C62" t="s">
+        <v>65</v>
+      </c>
+      <c r="D62" t="s">
+        <v>65</v>
+      </c>
+      <c r="E62" t="s">
+        <v>65</v>
+      </c>
+      <c r="F62" t="s">
+        <v>65</v>
+      </c>
+      <c r="G62" t="s">
+        <v>69</v>
+      </c>
+      <c r="H62" t="s">
+        <v>65</v>
+      </c>
+      <c r="I62" t="s">
+        <v>64</v>
+      </c>
+      <c r="J62" t="s">
+        <v>65</v>
+      </c>
+      <c r="K62" t="s">
+        <v>65</v>
+      </c>
+      <c r="L62" t="s">
+        <v>65</v>
+      </c>
+      <c r="M62" t="s">
+        <v>65</v>
+      </c>
+      <c r="N62" t="s">
+        <v>65</v>
+      </c>
+      <c r="O62" t="s">
+        <v>65</v>
+      </c>
+      <c r="P62" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q62" t="s">
+        <v>65</v>
+      </c>
+      <c r="R62" t="s">
+        <v>64</v>
+      </c>
+      <c r="S62" t="s">
+        <v>65</v>
+      </c>
+      <c r="T62" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B62" s="5"/>
-      <c r="C62" s="5"/>
-      <c r="D62" s="5"/>
-      <c r="E62" s="5"/>
-      <c r="F62" s="5"/>
-      <c r="G62" s="5"/>
-      <c r="H62" s="5"/>
-      <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
-      <c r="K62" s="5"/>
-      <c r="L62" s="5"/>
-      <c r="M62" s="5"/>
-      <c r="N62" s="5"/>
-      <c r="O62" s="5"/>
-      <c r="P62" s="5"/>
-      <c r="Q62" s="5"/>
-      <c r="R62" s="5"/>
-      <c r="S62" s="5"/>
-      <c r="T62" s="5"/>
-    </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A63" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B63" t="s">
-        <v>65</v>
-      </c>
-      <c r="C63" t="s">
-        <v>65</v>
-      </c>
-      <c r="D63" t="s">
-        <v>65</v>
-      </c>
-      <c r="E63" t="s">
-        <v>65</v>
-      </c>
-      <c r="F63" t="s">
-        <v>65</v>
-      </c>
-      <c r="G63" t="s">
-        <v>65</v>
-      </c>
-      <c r="H63" t="s">
-        <v>64</v>
-      </c>
-      <c r="I63" t="s">
-        <v>64</v>
-      </c>
-      <c r="J63" t="s">
-        <v>64</v>
-      </c>
-      <c r="K63" t="s">
-        <v>65</v>
-      </c>
-      <c r="L63" t="s">
-        <v>65</v>
-      </c>
-      <c r="M63" t="s">
-        <v>65</v>
-      </c>
-      <c r="N63" t="s">
-        <v>70</v>
-      </c>
-      <c r="O63" t="s">
-        <v>65</v>
-      </c>
-      <c r="P63" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q63" t="s">
-        <v>65</v>
-      </c>
-      <c r="R63" t="s">
-        <v>68</v>
-      </c>
-      <c r="S63" t="s">
-        <v>65</v>
-      </c>
-      <c r="T63" t="s">
-        <v>65</v>
-      </c>
+      <c r="B63" s="5"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="K63" s="5"/>
+      <c r="L63" s="5"/>
+      <c r="M63" s="5"/>
+      <c r="N63" s="5"/>
+      <c r="O63" s="5"/>
+      <c r="P63" s="5"/>
+      <c r="Q63" s="5"/>
+      <c r="R63" s="5"/>
+      <c r="S63" s="5"/>
+      <c r="T63" s="5"/>
     </row>
     <row r="64" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="B64" t="s">
         <v>65</v>
@@ -4126,7 +4128,7 @@
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B65" t="s">
         <v>65</v>
@@ -4150,10 +4152,10 @@
         <v>64</v>
       </c>
       <c r="I65" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J65" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K65" t="s">
         <v>65</v>
@@ -4187,174 +4189,214 @@
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A66" s="5" t="s">
+      <c r="A66" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B66" t="s">
+        <v>65</v>
+      </c>
+      <c r="C66" t="s">
+        <v>65</v>
+      </c>
+      <c r="D66" t="s">
+        <v>65</v>
+      </c>
+      <c r="E66" t="s">
+        <v>65</v>
+      </c>
+      <c r="F66" t="s">
+        <v>65</v>
+      </c>
+      <c r="G66" t="s">
+        <v>65</v>
+      </c>
+      <c r="H66" t="s">
+        <v>64</v>
+      </c>
+      <c r="I66" t="s">
+        <v>66</v>
+      </c>
+      <c r="J66" t="s">
+        <v>66</v>
+      </c>
+      <c r="K66" t="s">
+        <v>65</v>
+      </c>
+      <c r="L66" t="s">
+        <v>65</v>
+      </c>
+      <c r="M66" t="s">
+        <v>65</v>
+      </c>
+      <c r="N66" t="s">
+        <v>70</v>
+      </c>
+      <c r="O66" t="s">
+        <v>65</v>
+      </c>
+      <c r="P66" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q66" t="s">
+        <v>65</v>
+      </c>
+      <c r="R66" t="s">
+        <v>68</v>
+      </c>
+      <c r="S66" t="s">
+        <v>65</v>
+      </c>
+      <c r="T66" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A67" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B66" s="5"/>
-      <c r="C66" s="5"/>
-      <c r="D66" s="5"/>
-      <c r="E66" s="5"/>
-      <c r="F66" s="5"/>
-      <c r="G66" s="5"/>
-      <c r="H66" s="5"/>
-      <c r="I66" s="5"/>
-      <c r="J66" s="5"/>
-      <c r="K66" s="5"/>
-      <c r="L66" s="5"/>
-      <c r="M66" s="5"/>
-      <c r="N66" s="5"/>
-      <c r="O66" s="5"/>
-      <c r="P66" s="5"/>
-      <c r="Q66" s="5"/>
-      <c r="R66" s="5"/>
-      <c r="S66" s="5"/>
-      <c r="T66" s="5"/>
-    </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A67" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B67" t="s">
-        <v>65</v>
-      </c>
-      <c r="C67" t="s">
-        <v>65</v>
-      </c>
-      <c r="D67" t="s">
-        <v>65</v>
-      </c>
-      <c r="E67" t="s">
-        <v>65</v>
-      </c>
-      <c r="F67" t="s">
-        <v>65</v>
-      </c>
-      <c r="G67" t="s">
-        <v>65</v>
-      </c>
-      <c r="H67" t="s">
-        <v>64</v>
-      </c>
-      <c r="I67" t="s">
-        <v>64</v>
-      </c>
-      <c r="J67" t="s">
-        <v>64</v>
-      </c>
-      <c r="K67" t="s">
-        <v>65</v>
-      </c>
-      <c r="L67" t="s">
-        <v>65</v>
-      </c>
-      <c r="M67" t="s">
-        <v>65</v>
-      </c>
-      <c r="N67" t="s">
-        <v>70</v>
-      </c>
-      <c r="O67" t="s">
-        <v>65</v>
-      </c>
-      <c r="P67" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q67" t="s">
-        <v>65</v>
-      </c>
-      <c r="R67" t="s">
-        <v>64</v>
-      </c>
-      <c r="S67" t="s">
-        <v>65</v>
-      </c>
-      <c r="T67" t="s">
-        <v>69</v>
-      </c>
+      <c r="B67" s="5"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="5"/>
+      <c r="G67" s="5"/>
+      <c r="H67" s="5"/>
+      <c r="I67" s="5"/>
+      <c r="J67" s="5"/>
+      <c r="K67" s="5"/>
+      <c r="L67" s="5"/>
+      <c r="M67" s="5"/>
+      <c r="N67" s="5"/>
+      <c r="O67" s="5"/>
+      <c r="P67" s="5"/>
+      <c r="Q67" s="5"/>
+      <c r="R67" s="5"/>
+      <c r="S67" s="5"/>
+      <c r="T67" s="5"/>
     </row>
     <row r="68" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B68" t="s">
+        <v>65</v>
+      </c>
+      <c r="C68" t="s">
+        <v>65</v>
+      </c>
+      <c r="D68" t="s">
+        <v>65</v>
+      </c>
+      <c r="E68" t="s">
+        <v>65</v>
+      </c>
+      <c r="F68" t="s">
+        <v>65</v>
+      </c>
+      <c r="G68" t="s">
+        <v>65</v>
+      </c>
+      <c r="H68" t="s">
+        <v>64</v>
+      </c>
+      <c r="I68" t="s">
+        <v>64</v>
+      </c>
+      <c r="J68" t="s">
+        <v>64</v>
+      </c>
+      <c r="K68" t="s">
+        <v>65</v>
+      </c>
+      <c r="L68" t="s">
+        <v>65</v>
+      </c>
+      <c r="M68" t="s">
+        <v>65</v>
+      </c>
+      <c r="N68" t="s">
+        <v>70</v>
+      </c>
+      <c r="O68" t="s">
+        <v>65</v>
+      </c>
+      <c r="P68" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q68" t="s">
+        <v>65</v>
+      </c>
+      <c r="R68" t="s">
+        <v>64</v>
+      </c>
+      <c r="S68" t="s">
+        <v>65</v>
+      </c>
+      <c r="T68" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B68" t="s">
-        <v>65</v>
-      </c>
-      <c r="C68" t="s">
-        <v>65</v>
-      </c>
-      <c r="D68" t="s">
-        <v>65</v>
-      </c>
-      <c r="E68" t="s">
-        <v>65</v>
-      </c>
-      <c r="F68" t="s">
-        <v>65</v>
-      </c>
-      <c r="G68" t="s">
-        <v>65</v>
-      </c>
-      <c r="H68" t="s">
-        <v>64</v>
-      </c>
-      <c r="I68" t="s">
-        <v>64</v>
-      </c>
-      <c r="J68" t="s">
-        <v>64</v>
-      </c>
-      <c r="K68" t="s">
-        <v>65</v>
-      </c>
-      <c r="L68" t="s">
-        <v>65</v>
-      </c>
-      <c r="M68" t="s">
-        <v>65</v>
-      </c>
-      <c r="N68" t="s">
-        <v>70</v>
-      </c>
-      <c r="O68" t="s">
-        <v>65</v>
-      </c>
-      <c r="P68" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q68" t="s">
-        <v>65</v>
-      </c>
-      <c r="R68" t="s">
-        <v>64</v>
-      </c>
-      <c r="S68" t="s">
-        <v>65</v>
-      </c>
-      <c r="T68" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A69" s="7"/>
-      <c r="B69" s="7"/>
-      <c r="C69" s="7"/>
-      <c r="D69" s="7"/>
-      <c r="E69" s="7"/>
-      <c r="F69" s="7"/>
-      <c r="G69" s="7"/>
-      <c r="H69" s="7"/>
-      <c r="I69" s="7"/>
-      <c r="J69" s="7"/>
-      <c r="K69" s="7"/>
-      <c r="L69" s="7"/>
-      <c r="M69" s="7"/>
-      <c r="N69" s="7"/>
-      <c r="O69" s="7"/>
-      <c r="P69" s="7"/>
-      <c r="Q69" s="7"/>
-      <c r="R69" s="7"/>
-      <c r="S69" s="7"/>
-      <c r="T69" s="7"/>
+      <c r="B69" t="s">
+        <v>65</v>
+      </c>
+      <c r="C69" t="s">
+        <v>65</v>
+      </c>
+      <c r="D69" t="s">
+        <v>65</v>
+      </c>
+      <c r="E69" t="s">
+        <v>65</v>
+      </c>
+      <c r="F69" t="s">
+        <v>65</v>
+      </c>
+      <c r="G69" t="s">
+        <v>65</v>
+      </c>
+      <c r="H69" t="s">
+        <v>64</v>
+      </c>
+      <c r="I69" t="s">
+        <v>64</v>
+      </c>
+      <c r="J69" t="s">
+        <v>64</v>
+      </c>
+      <c r="K69" t="s">
+        <v>65</v>
+      </c>
+      <c r="L69" t="s">
+        <v>65</v>
+      </c>
+      <c r="M69" t="s">
+        <v>65</v>
+      </c>
+      <c r="N69" t="s">
+        <v>70</v>
+      </c>
+      <c r="O69" t="s">
+        <v>65</v>
+      </c>
+      <c r="P69" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q69" t="s">
+        <v>65</v>
+      </c>
+      <c r="R69" t="s">
+        <v>64</v>
+      </c>
+      <c r="S69" t="s">
+        <v>65</v>
+      </c>
+      <c r="T69" t="s">
+        <v>69</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added class and class stat tables
</commit_message>
<xml_diff>
--- a/Documentation/CRUD Table.xlsx
+++ b/Documentation/CRUD Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dyfry\workspace\2026\DAT602-Project\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E2A387-E485-4B3F-A3CB-45B04935B674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CA1C611-3724-4BF4-9644-C4AF572D49DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1095" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1197" uniqueCount="92">
   <si>
     <t>Account</t>
   </si>
@@ -286,6 +286,21 @@
   </si>
   <si>
     <t>Combatant (FK)</t>
+  </si>
+  <si>
+    <t>Class (FK)</t>
+  </si>
+  <si>
+    <t>Class</t>
+  </si>
+  <si>
+    <t>Class_Statistic</t>
+  </si>
+  <si>
+    <t>ClassName (PK)</t>
+  </si>
+  <si>
+    <t>ClassName (PK) (FK)</t>
   </si>
 </sst>
 </file>
@@ -665,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T69"/>
+  <dimension ref="A1:T76"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.21875" customWidth="1"/>
@@ -1717,94 +1732,94 @@
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" t="s">
+        <v>65</v>
+      </c>
+      <c r="F20" t="s">
+        <v>65</v>
+      </c>
+      <c r="G20" t="s">
+        <v>65</v>
+      </c>
+      <c r="H20" t="s">
+        <v>65</v>
+      </c>
+      <c r="I20" t="s">
+        <v>65</v>
+      </c>
+      <c r="J20" t="s">
+        <v>65</v>
+      </c>
+      <c r="K20" t="s">
+        <v>65</v>
+      </c>
+      <c r="L20" t="s">
+        <v>65</v>
+      </c>
+      <c r="M20" t="s">
+        <v>65</v>
+      </c>
+      <c r="N20" t="s">
+        <v>70</v>
+      </c>
+      <c r="O20" t="s">
+        <v>65</v>
+      </c>
+      <c r="P20" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>65</v>
+      </c>
+      <c r="R20" t="s">
+        <v>69</v>
+      </c>
+      <c r="S20" t="s">
+        <v>65</v>
+      </c>
+      <c r="T20" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="5"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-      <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
-      <c r="K20" s="5"/>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
-      <c r="P20" s="5"/>
-      <c r="Q20" s="5"/>
-      <c r="R20" s="5"/>
-      <c r="S20" s="5"/>
-      <c r="T20" s="5"/>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A21" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" t="s">
-        <v>65</v>
-      </c>
-      <c r="C21" t="s">
-        <v>65</v>
-      </c>
-      <c r="D21" t="s">
-        <v>65</v>
-      </c>
-      <c r="E21" t="s">
-        <v>65</v>
-      </c>
-      <c r="F21" t="s">
-        <v>65</v>
-      </c>
-      <c r="G21" t="s">
-        <v>65</v>
-      </c>
-      <c r="H21" t="s">
-        <v>65</v>
-      </c>
-      <c r="I21" t="s">
-        <v>65</v>
-      </c>
-      <c r="J21" t="s">
-        <v>65</v>
-      </c>
-      <c r="K21" t="s">
-        <v>65</v>
-      </c>
-      <c r="L21" t="s">
-        <v>65</v>
-      </c>
-      <c r="M21" t="s">
-        <v>65</v>
-      </c>
-      <c r="N21" t="s">
-        <v>70</v>
-      </c>
-      <c r="O21" t="s">
-        <v>65</v>
-      </c>
-      <c r="P21" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q21" t="s">
-        <v>65</v>
-      </c>
-      <c r="R21" t="s">
-        <v>64</v>
-      </c>
-      <c r="S21" t="s">
-        <v>69</v>
-      </c>
-      <c r="T21" t="s">
-        <v>65</v>
-      </c>
+      <c r="B21" s="5"/>
+      <c r="C21" s="5"/>
+      <c r="D21" s="5"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
+      <c r="P21" s="5"/>
+      <c r="Q21" s="5"/>
+      <c r="R21" s="5"/>
+      <c r="S21" s="5"/>
+      <c r="T21" s="5"/>
     </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
         <v>65</v>
@@ -1866,7 +1881,7 @@
     </row>
     <row r="23" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B23" t="s">
         <v>65</v>
@@ -1927,94 +1942,94 @@
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B24" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" t="s">
+        <v>65</v>
+      </c>
+      <c r="D24" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F24" t="s">
+        <v>65</v>
+      </c>
+      <c r="G24" t="s">
+        <v>65</v>
+      </c>
+      <c r="H24" t="s">
+        <v>65</v>
+      </c>
+      <c r="I24" t="s">
+        <v>65</v>
+      </c>
+      <c r="J24" t="s">
+        <v>65</v>
+      </c>
+      <c r="K24" t="s">
+        <v>65</v>
+      </c>
+      <c r="L24" t="s">
+        <v>65</v>
+      </c>
+      <c r="M24" t="s">
+        <v>65</v>
+      </c>
+      <c r="N24" t="s">
+        <v>70</v>
+      </c>
+      <c r="O24" t="s">
+        <v>65</v>
+      </c>
+      <c r="P24" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>65</v>
+      </c>
+      <c r="R24" t="s">
+        <v>64</v>
+      </c>
+      <c r="S24" t="s">
+        <v>69</v>
+      </c>
+      <c r="T24" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
-      <c r="P24" s="5"/>
-      <c r="Q24" s="5"/>
-      <c r="R24" s="5"/>
-      <c r="S24" s="5"/>
-      <c r="T24" s="5"/>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A25" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B25" t="s">
-        <v>65</v>
-      </c>
-      <c r="C25" t="s">
-        <v>65</v>
-      </c>
-      <c r="D25" t="s">
-        <v>65</v>
-      </c>
-      <c r="E25" t="s">
-        <v>65</v>
-      </c>
-      <c r="F25" t="s">
-        <v>65</v>
-      </c>
-      <c r="G25" t="s">
-        <v>65</v>
-      </c>
-      <c r="H25" t="s">
-        <v>65</v>
-      </c>
-      <c r="I25" t="s">
-        <v>65</v>
-      </c>
-      <c r="J25" t="s">
-        <v>65</v>
-      </c>
-      <c r="K25" t="s">
-        <v>65</v>
-      </c>
-      <c r="L25" t="s">
-        <v>65</v>
-      </c>
-      <c r="M25" t="s">
-        <v>65</v>
-      </c>
-      <c r="N25" t="s">
-        <v>70</v>
-      </c>
-      <c r="O25" t="s">
-        <v>65</v>
-      </c>
-      <c r="P25" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q25" t="s">
-        <v>65</v>
-      </c>
-      <c r="R25" t="s">
-        <v>64</v>
-      </c>
-      <c r="S25" t="s">
-        <v>65</v>
-      </c>
-      <c r="T25" t="s">
-        <v>69</v>
-      </c>
+      <c r="B25" s="5"/>
+      <c r="C25" s="5"/>
+      <c r="D25" s="5"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+      <c r="N25" s="5"/>
+      <c r="O25" s="5"/>
+      <c r="P25" s="5"/>
+      <c r="Q25" s="5"/>
+      <c r="R25" s="5"/>
+      <c r="S25" s="5"/>
+      <c r="T25" s="5"/>
     </row>
     <row r="26" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B26" t="s">
         <v>65</v>
@@ -2076,7 +2091,7 @@
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B27" t="s">
         <v>65</v>
@@ -2137,94 +2152,94 @@
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" t="s">
+        <v>65</v>
+      </c>
+      <c r="G28" t="s">
+        <v>65</v>
+      </c>
+      <c r="H28" t="s">
+        <v>65</v>
+      </c>
+      <c r="I28" t="s">
+        <v>65</v>
+      </c>
+      <c r="J28" t="s">
+        <v>65</v>
+      </c>
+      <c r="K28" t="s">
+        <v>65</v>
+      </c>
+      <c r="L28" t="s">
+        <v>65</v>
+      </c>
+      <c r="M28" t="s">
+        <v>65</v>
+      </c>
+      <c r="N28" t="s">
+        <v>70</v>
+      </c>
+      <c r="O28" t="s">
+        <v>65</v>
+      </c>
+      <c r="P28" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q28" t="s">
+        <v>65</v>
+      </c>
+      <c r="R28" t="s">
+        <v>64</v>
+      </c>
+      <c r="S28" t="s">
+        <v>65</v>
+      </c>
+      <c r="T28" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="5"/>
-      <c r="O28" s="5"/>
-      <c r="P28" s="5"/>
-      <c r="Q28" s="5"/>
-      <c r="R28" s="5"/>
-      <c r="S28" s="5"/>
-      <c r="T28" s="5"/>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A29" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="B29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C29" t="s">
-        <v>65</v>
-      </c>
-      <c r="D29" t="s">
-        <v>65</v>
-      </c>
-      <c r="E29" t="s">
-        <v>65</v>
-      </c>
-      <c r="F29" t="s">
-        <v>65</v>
-      </c>
-      <c r="G29" t="s">
-        <v>65</v>
-      </c>
-      <c r="H29" t="s">
-        <v>69</v>
-      </c>
-      <c r="I29" t="s">
-        <v>65</v>
-      </c>
-      <c r="J29" t="s">
-        <v>65</v>
-      </c>
-      <c r="K29" t="s">
-        <v>65</v>
-      </c>
-      <c r="L29" t="s">
-        <v>69</v>
-      </c>
-      <c r="M29" t="s">
-        <v>64</v>
-      </c>
-      <c r="N29" t="s">
-        <v>70</v>
-      </c>
-      <c r="O29" t="s">
-        <v>65</v>
-      </c>
-      <c r="P29" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q29" t="s">
-        <v>65</v>
-      </c>
-      <c r="R29" t="s">
-        <v>64</v>
-      </c>
-      <c r="S29" t="s">
-        <v>65</v>
-      </c>
-      <c r="T29" t="s">
-        <v>65</v>
-      </c>
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+      <c r="O29" s="5"/>
+      <c r="P29" s="5"/>
+      <c r="Q29" s="5"/>
+      <c r="R29" s="5"/>
+      <c r="S29" s="5"/>
+      <c r="T29" s="5"/>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="B30" t="s">
         <v>65</v>
@@ -2286,7 +2301,7 @@
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B31" t="s">
         <v>65</v>
@@ -2347,94 +2362,94 @@
       </c>
     </row>
     <row r="32" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B32" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" t="s">
+        <v>65</v>
+      </c>
+      <c r="F32" t="s">
+        <v>65</v>
+      </c>
+      <c r="G32" t="s">
+        <v>65</v>
+      </c>
+      <c r="H32" t="s">
+        <v>69</v>
+      </c>
+      <c r="I32" t="s">
+        <v>65</v>
+      </c>
+      <c r="J32" t="s">
+        <v>65</v>
+      </c>
+      <c r="K32" t="s">
+        <v>65</v>
+      </c>
+      <c r="L32" t="s">
+        <v>69</v>
+      </c>
+      <c r="M32" t="s">
+        <v>64</v>
+      </c>
+      <c r="N32" t="s">
+        <v>70</v>
+      </c>
+      <c r="O32" t="s">
+        <v>65</v>
+      </c>
+      <c r="P32" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>65</v>
+      </c>
+      <c r="R32" t="s">
+        <v>64</v>
+      </c>
+      <c r="S32" t="s">
+        <v>65</v>
+      </c>
+      <c r="T32" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="5"/>
-      <c r="O32" s="5"/>
-      <c r="P32" s="5"/>
-      <c r="Q32" s="5"/>
-      <c r="R32" s="5"/>
-      <c r="S32" s="5"/>
-      <c r="T32" s="5"/>
-    </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A33" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B33" t="s">
-        <v>65</v>
-      </c>
-      <c r="C33" t="s">
-        <v>65</v>
-      </c>
-      <c r="D33" t="s">
-        <v>65</v>
-      </c>
-      <c r="E33" t="s">
-        <v>65</v>
-      </c>
-      <c r="F33" t="s">
-        <v>64</v>
-      </c>
-      <c r="G33" t="s">
-        <v>64</v>
-      </c>
-      <c r="H33" t="s">
-        <v>64</v>
-      </c>
-      <c r="I33" t="s">
-        <v>65</v>
-      </c>
-      <c r="J33" t="s">
-        <v>64</v>
-      </c>
-      <c r="K33" t="s">
-        <v>65</v>
-      </c>
-      <c r="L33" t="s">
-        <v>64</v>
-      </c>
-      <c r="M33" t="s">
-        <v>64</v>
-      </c>
-      <c r="N33" t="s">
-        <v>70</v>
-      </c>
-      <c r="O33" t="s">
-        <v>65</v>
-      </c>
-      <c r="P33" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q33" t="s">
-        <v>65</v>
-      </c>
-      <c r="R33" t="s">
-        <v>64</v>
-      </c>
-      <c r="S33" t="s">
-        <v>65</v>
-      </c>
-      <c r="T33" t="s">
-        <v>69</v>
-      </c>
+      <c r="B33" s="5"/>
+      <c r="C33" s="5"/>
+      <c r="D33" s="5"/>
+      <c r="E33" s="5"/>
+      <c r="F33" s="5"/>
+      <c r="G33" s="5"/>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+      <c r="N33" s="5"/>
+      <c r="O33" s="5"/>
+      <c r="P33" s="5"/>
+      <c r="Q33" s="5"/>
+      <c r="R33" s="5"/>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B34" t="s">
         <v>65</v>
@@ -2452,25 +2467,25 @@
         <v>64</v>
       </c>
       <c r="G34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I34" t="s">
         <v>65</v>
       </c>
       <c r="J34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="K34" t="s">
         <v>65</v>
       </c>
       <c r="L34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="M34" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="N34" t="s">
         <v>70</v>
@@ -2496,7 +2511,7 @@
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B35" t="s">
         <v>65</v>
@@ -2558,155 +2573,155 @@
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" t="s">
+        <v>65</v>
+      </c>
+      <c r="D36" t="s">
+        <v>65</v>
+      </c>
+      <c r="E36" t="s">
+        <v>65</v>
+      </c>
+      <c r="F36" t="s">
+        <v>64</v>
+      </c>
+      <c r="G36" t="s">
+        <v>65</v>
+      </c>
+      <c r="H36" t="s">
+        <v>65</v>
+      </c>
+      <c r="I36" t="s">
+        <v>65</v>
+      </c>
+      <c r="J36" t="s">
+        <v>65</v>
+      </c>
+      <c r="K36" t="s">
+        <v>65</v>
+      </c>
+      <c r="L36" t="s">
+        <v>65</v>
+      </c>
+      <c r="M36" t="s">
+        <v>65</v>
+      </c>
+      <c r="N36" t="s">
+        <v>70</v>
+      </c>
+      <c r="O36" t="s">
+        <v>65</v>
+      </c>
+      <c r="P36" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>65</v>
+      </c>
+      <c r="R36" t="s">
+        <v>64</v>
+      </c>
+      <c r="S36" t="s">
+        <v>65</v>
+      </c>
+      <c r="T36" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B36" t="s">
-        <v>65</v>
-      </c>
-      <c r="C36" t="s">
-        <v>65</v>
-      </c>
-      <c r="D36" t="s">
-        <v>65</v>
-      </c>
-      <c r="E36" t="s">
-        <v>65</v>
-      </c>
-      <c r="F36" t="s">
-        <v>64</v>
-      </c>
-      <c r="G36" t="s">
-        <v>65</v>
-      </c>
-      <c r="H36" t="s">
-        <v>65</v>
-      </c>
-      <c r="I36" t="s">
-        <v>65</v>
-      </c>
-      <c r="J36" t="s">
-        <v>65</v>
-      </c>
-      <c r="K36" t="s">
-        <v>65</v>
-      </c>
-      <c r="L36" t="s">
-        <v>65</v>
-      </c>
-      <c r="M36" t="s">
-        <v>65</v>
-      </c>
-      <c r="N36" t="s">
-        <v>70</v>
-      </c>
-      <c r="O36" t="s">
-        <v>65</v>
-      </c>
-      <c r="P36" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>65</v>
-      </c>
-      <c r="R36" t="s">
-        <v>64</v>
-      </c>
-      <c r="S36" t="s">
-        <v>65</v>
-      </c>
-      <c r="T36" t="s">
+      <c r="B37" t="s">
+        <v>65</v>
+      </c>
+      <c r="C37" t="s">
+        <v>65</v>
+      </c>
+      <c r="D37" t="s">
+        <v>65</v>
+      </c>
+      <c r="E37" t="s">
+        <v>65</v>
+      </c>
+      <c r="F37" t="s">
+        <v>64</v>
+      </c>
+      <c r="G37" t="s">
+        <v>65</v>
+      </c>
+      <c r="H37" t="s">
+        <v>65</v>
+      </c>
+      <c r="I37" t="s">
+        <v>65</v>
+      </c>
+      <c r="J37" t="s">
+        <v>65</v>
+      </c>
+      <c r="K37" t="s">
+        <v>65</v>
+      </c>
+      <c r="L37" t="s">
+        <v>65</v>
+      </c>
+      <c r="M37" t="s">
+        <v>65</v>
+      </c>
+      <c r="N37" t="s">
+        <v>70</v>
+      </c>
+      <c r="O37" t="s">
+        <v>65</v>
+      </c>
+      <c r="P37" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>65</v>
+      </c>
+      <c r="R37" t="s">
+        <v>64</v>
+      </c>
+      <c r="S37" t="s">
+        <v>65</v>
+      </c>
+      <c r="T37" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A37" s="5" t="s">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B37" s="5"/>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="E37" s="5"/>
-      <c r="F37" s="5"/>
-      <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-      <c r="K37" s="5"/>
-      <c r="L37" s="5"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="5"/>
-      <c r="O37" s="5"/>
-      <c r="P37" s="5"/>
-      <c r="Q37" s="5"/>
-      <c r="R37" s="5"/>
-      <c r="S37" s="5"/>
-      <c r="T37" s="5"/>
-    </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B38" t="s">
-        <v>65</v>
-      </c>
-      <c r="C38" t="s">
-        <v>65</v>
-      </c>
-      <c r="D38" t="s">
-        <v>65</v>
-      </c>
-      <c r="E38" t="s">
-        <v>65</v>
-      </c>
-      <c r="F38" t="s">
-        <v>65</v>
-      </c>
-      <c r="G38" t="s">
-        <v>69</v>
-      </c>
-      <c r="H38" t="s">
-        <v>64</v>
-      </c>
-      <c r="I38" t="s">
-        <v>64</v>
-      </c>
-      <c r="J38" t="s">
-        <v>69</v>
-      </c>
-      <c r="K38" t="s">
-        <v>65</v>
-      </c>
-      <c r="L38" t="s">
-        <v>65</v>
-      </c>
-      <c r="M38" t="s">
-        <v>68</v>
-      </c>
-      <c r="N38" t="s">
-        <v>70</v>
-      </c>
-      <c r="O38" t="s">
-        <v>65</v>
-      </c>
-      <c r="P38" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>65</v>
-      </c>
-      <c r="R38" t="s">
-        <v>64</v>
-      </c>
-      <c r="S38" t="s">
-        <v>65</v>
-      </c>
-      <c r="T38" t="s">
-        <v>65</v>
-      </c>
+      <c r="B38" s="5"/>
+      <c r="C38" s="5"/>
+      <c r="D38" s="5"/>
+      <c r="E38" s="5"/>
+      <c r="F38" s="5"/>
+      <c r="G38" s="5"/>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+      <c r="N38" s="5"/>
+      <c r="O38" s="5"/>
+      <c r="P38" s="5"/>
+      <c r="Q38" s="5"/>
+      <c r="R38" s="5"/>
+      <c r="S38" s="5"/>
+      <c r="T38" s="5"/>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>45</v>
+        <v>82</v>
       </c>
       <c r="B39" t="s">
         <v>65</v>
@@ -2768,7 +2783,7 @@
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="B40" t="s">
         <v>65</v>
@@ -2830,7 +2845,7 @@
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B41" t="s">
         <v>65</v>
@@ -2848,16 +2863,16 @@
         <v>65</v>
       </c>
       <c r="G41" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="H41" t="s">
         <v>64</v>
       </c>
       <c r="I41" t="s">
+        <v>64</v>
+      </c>
+      <c r="J41" t="s">
         <v>69</v>
-      </c>
-      <c r="J41" t="s">
-        <v>65</v>
       </c>
       <c r="K41" t="s">
         <v>65</v>
@@ -2891,94 +2906,94 @@
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B42" t="s">
+        <v>65</v>
+      </c>
+      <c r="C42" t="s">
+        <v>65</v>
+      </c>
+      <c r="D42" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" t="s">
+        <v>65</v>
+      </c>
+      <c r="F42" t="s">
+        <v>65</v>
+      </c>
+      <c r="G42" t="s">
+        <v>65</v>
+      </c>
+      <c r="H42" t="s">
+        <v>64</v>
+      </c>
+      <c r="I42" t="s">
+        <v>69</v>
+      </c>
+      <c r="J42" t="s">
+        <v>65</v>
+      </c>
+      <c r="K42" t="s">
+        <v>65</v>
+      </c>
+      <c r="L42" t="s">
+        <v>65</v>
+      </c>
+      <c r="M42" t="s">
+        <v>68</v>
+      </c>
+      <c r="N42" t="s">
+        <v>70</v>
+      </c>
+      <c r="O42" t="s">
+        <v>65</v>
+      </c>
+      <c r="P42" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q42" t="s">
+        <v>65</v>
+      </c>
+      <c r="R42" t="s">
+        <v>64</v>
+      </c>
+      <c r="S42" t="s">
+        <v>65</v>
+      </c>
+      <c r="T42" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B42" s="5"/>
-      <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="5"/>
-      <c r="F42" s="5"/>
-      <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-      <c r="I42" s="5"/>
-      <c r="J42" s="5"/>
-      <c r="K42" s="5"/>
-      <c r="L42" s="5"/>
-      <c r="M42" s="5"/>
-      <c r="N42" s="5"/>
-      <c r="O42" s="5"/>
-      <c r="P42" s="5"/>
-      <c r="Q42" s="5"/>
-      <c r="R42" s="5"/>
-      <c r="S42" s="5"/>
-      <c r="T42" s="5"/>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A43" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B43" t="s">
-        <v>65</v>
-      </c>
-      <c r="C43" t="s">
-        <v>65</v>
-      </c>
-      <c r="D43" t="s">
-        <v>65</v>
-      </c>
-      <c r="E43" t="s">
-        <v>65</v>
-      </c>
-      <c r="F43" t="s">
-        <v>65</v>
-      </c>
-      <c r="G43" t="s">
-        <v>68</v>
-      </c>
-      <c r="H43" t="s">
-        <v>65</v>
-      </c>
-      <c r="I43" t="s">
-        <v>64</v>
-      </c>
-      <c r="J43" t="s">
-        <v>64</v>
-      </c>
-      <c r="K43" t="s">
-        <v>65</v>
-      </c>
-      <c r="L43" t="s">
-        <v>65</v>
-      </c>
-      <c r="M43" t="s">
-        <v>65</v>
-      </c>
-      <c r="N43" t="s">
-        <v>65</v>
-      </c>
-      <c r="O43" t="s">
-        <v>65</v>
-      </c>
-      <c r="P43" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q43" t="s">
-        <v>65</v>
-      </c>
-      <c r="R43" t="s">
-        <v>64</v>
-      </c>
-      <c r="S43" t="s">
-        <v>65</v>
-      </c>
-      <c r="T43" t="s">
-        <v>65</v>
-      </c>
+      <c r="B43" s="5"/>
+      <c r="C43" s="5"/>
+      <c r="D43" s="5"/>
+      <c r="E43" s="5"/>
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="5"/>
+      <c r="L43" s="5"/>
+      <c r="M43" s="5"/>
+      <c r="N43" s="5"/>
+      <c r="O43" s="5"/>
+      <c r="P43" s="5"/>
+      <c r="Q43" s="5"/>
+      <c r="R43" s="5"/>
+      <c r="S43" s="5"/>
+      <c r="T43" s="5"/>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="B44" t="s">
         <v>65</v>
@@ -3040,7 +3055,7 @@
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" t="s">
         <v>65</v>
@@ -3102,7 +3117,7 @@
     </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" t="s">
         <v>65</v>
@@ -3164,7 +3179,7 @@
     </row>
     <row r="47" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" t="s">
         <v>65</v>
@@ -3226,7 +3241,7 @@
     </row>
     <row r="48" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B48" t="s">
         <v>65</v>
@@ -3288,7 +3303,7 @@
     </row>
     <row r="49" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B49" t="s">
         <v>65</v>
@@ -3350,7 +3365,7 @@
     </row>
     <row r="50" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B50" t="s">
         <v>65</v>
@@ -3411,94 +3426,94 @@
       </c>
     </row>
     <row r="51" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B51" t="s">
+        <v>65</v>
+      </c>
+      <c r="C51" t="s">
+        <v>65</v>
+      </c>
+      <c r="D51" t="s">
+        <v>65</v>
+      </c>
+      <c r="E51" t="s">
+        <v>65</v>
+      </c>
+      <c r="F51" t="s">
+        <v>65</v>
+      </c>
+      <c r="G51" t="s">
+        <v>68</v>
+      </c>
+      <c r="H51" t="s">
+        <v>65</v>
+      </c>
+      <c r="I51" t="s">
+        <v>64</v>
+      </c>
+      <c r="J51" t="s">
+        <v>64</v>
+      </c>
+      <c r="K51" t="s">
+        <v>65</v>
+      </c>
+      <c r="L51" t="s">
+        <v>65</v>
+      </c>
+      <c r="M51" t="s">
+        <v>65</v>
+      </c>
+      <c r="N51" t="s">
+        <v>65</v>
+      </c>
+      <c r="O51" t="s">
+        <v>65</v>
+      </c>
+      <c r="P51" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q51" t="s">
+        <v>65</v>
+      </c>
+      <c r="R51" t="s">
+        <v>64</v>
+      </c>
+      <c r="S51" t="s">
+        <v>65</v>
+      </c>
+      <c r="T51" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B51" s="5"/>
-      <c r="C51" s="5"/>
-      <c r="D51" s="5"/>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
-      <c r="K51" s="5"/>
-      <c r="L51" s="5"/>
-      <c r="M51" s="5"/>
-      <c r="N51" s="5"/>
-      <c r="O51" s="5"/>
-      <c r="P51" s="5"/>
-      <c r="Q51" s="5"/>
-      <c r="R51" s="5"/>
-      <c r="S51" s="5"/>
-      <c r="T51" s="5"/>
-    </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A52" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B52" t="s">
-        <v>65</v>
-      </c>
-      <c r="C52" t="s">
-        <v>65</v>
-      </c>
-      <c r="D52" t="s">
-        <v>65</v>
-      </c>
-      <c r="E52" t="s">
-        <v>65</v>
-      </c>
-      <c r="F52" t="s">
-        <v>65</v>
-      </c>
-      <c r="G52" t="s">
-        <v>65</v>
-      </c>
-      <c r="H52" t="s">
-        <v>65</v>
-      </c>
-      <c r="I52" t="s">
-        <v>69</v>
-      </c>
-      <c r="J52" t="s">
-        <v>64</v>
-      </c>
-      <c r="K52" t="s">
-        <v>65</v>
-      </c>
-      <c r="L52" t="s">
-        <v>64</v>
-      </c>
-      <c r="M52" t="s">
-        <v>65</v>
-      </c>
-      <c r="N52" t="s">
-        <v>70</v>
-      </c>
-      <c r="O52" t="s">
-        <v>65</v>
-      </c>
-      <c r="P52" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q52" t="s">
-        <v>65</v>
-      </c>
-      <c r="R52" t="s">
-        <v>64</v>
-      </c>
-      <c r="S52" t="s">
-        <v>65</v>
-      </c>
-      <c r="T52" t="s">
-        <v>65</v>
-      </c>
+      <c r="B52" s="5"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="5"/>
+      <c r="E52" s="5"/>
+      <c r="F52" s="5"/>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+      <c r="N52" s="5"/>
+      <c r="O52" s="5"/>
+      <c r="P52" s="5"/>
+      <c r="Q52" s="5"/>
+      <c r="R52" s="5"/>
+      <c r="S52" s="5"/>
+      <c r="T52" s="5"/>
     </row>
     <row r="53" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="B53" t="s">
         <v>65</v>
@@ -3528,7 +3543,7 @@
         <v>64</v>
       </c>
       <c r="K53" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="L53" t="s">
         <v>64</v>
@@ -3560,7 +3575,7 @@
     </row>
     <row r="54" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="B54" t="s">
         <v>65</v>
@@ -3622,7 +3637,7 @@
     </row>
     <row r="55" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="B55" t="s">
         <v>65</v>
@@ -3649,128 +3664,128 @@
         <v>69</v>
       </c>
       <c r="J55" t="s">
+        <v>64</v>
+      </c>
+      <c r="K55" t="s">
+        <v>64</v>
+      </c>
+      <c r="L55" t="s">
+        <v>64</v>
+      </c>
+      <c r="M55" t="s">
+        <v>65</v>
+      </c>
+      <c r="N55" t="s">
+        <v>70</v>
+      </c>
+      <c r="O55" t="s">
+        <v>65</v>
+      </c>
+      <c r="P55" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q55" t="s">
+        <v>65</v>
+      </c>
+      <c r="R55" t="s">
+        <v>64</v>
+      </c>
+      <c r="S55" t="s">
+        <v>65</v>
+      </c>
+      <c r="T55" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B56" t="s">
+        <v>65</v>
+      </c>
+      <c r="C56" t="s">
+        <v>65</v>
+      </c>
+      <c r="D56" t="s">
+        <v>65</v>
+      </c>
+      <c r="E56" t="s">
+        <v>65</v>
+      </c>
+      <c r="F56" t="s">
+        <v>65</v>
+      </c>
+      <c r="G56" t="s">
+        <v>65</v>
+      </c>
+      <c r="H56" t="s">
+        <v>65</v>
+      </c>
+      <c r="I56" t="s">
+        <v>69</v>
+      </c>
+      <c r="J56" t="s">
         <v>66</v>
       </c>
-      <c r="K55" t="s">
-        <v>64</v>
-      </c>
-      <c r="L55" t="s">
+      <c r="K56" t="s">
+        <v>64</v>
+      </c>
+      <c r="L56" t="s">
         <v>66</v>
       </c>
-      <c r="M55" t="s">
-        <v>65</v>
-      </c>
-      <c r="N55" t="s">
-        <v>70</v>
-      </c>
-      <c r="O55" t="s">
-        <v>65</v>
-      </c>
-      <c r="P55" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q55" t="s">
-        <v>65</v>
-      </c>
-      <c r="R55" t="s">
-        <v>64</v>
-      </c>
-      <c r="S55" t="s">
-        <v>65</v>
-      </c>
-      <c r="T55" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A56" s="5" t="s">
+      <c r="M56" t="s">
+        <v>65</v>
+      </c>
+      <c r="N56" t="s">
+        <v>70</v>
+      </c>
+      <c r="O56" t="s">
+        <v>65</v>
+      </c>
+      <c r="P56" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q56" t="s">
+        <v>65</v>
+      </c>
+      <c r="R56" t="s">
+        <v>64</v>
+      </c>
+      <c r="S56" t="s">
+        <v>65</v>
+      </c>
+      <c r="T56" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B56" s="5"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
-      <c r="E56" s="5"/>
-      <c r="F56" s="5"/>
-      <c r="G56" s="5"/>
-      <c r="H56" s="5"/>
-      <c r="I56" s="5"/>
-      <c r="J56" s="5"/>
-      <c r="K56" s="5"/>
-      <c r="L56" s="5"/>
-      <c r="M56" s="5"/>
-      <c r="N56" s="5"/>
-      <c r="O56" s="5"/>
-      <c r="P56" s="5"/>
-      <c r="Q56" s="5"/>
-      <c r="R56" s="5"/>
-      <c r="S56" s="5"/>
-      <c r="T56" s="5"/>
-    </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A57" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="B57" t="s">
-        <v>65</v>
-      </c>
-      <c r="C57" t="s">
-        <v>65</v>
-      </c>
-      <c r="D57" t="s">
-        <v>65</v>
-      </c>
-      <c r="E57" t="s">
-        <v>65</v>
-      </c>
-      <c r="F57" t="s">
-        <v>65</v>
-      </c>
-      <c r="G57" t="s">
-        <v>69</v>
-      </c>
-      <c r="H57" t="s">
-        <v>65</v>
-      </c>
-      <c r="I57" t="s">
-        <v>64</v>
-      </c>
-      <c r="J57" t="s">
-        <v>65</v>
-      </c>
-      <c r="K57" t="s">
-        <v>65</v>
-      </c>
-      <c r="L57" t="s">
-        <v>65</v>
-      </c>
-      <c r="M57" t="s">
-        <v>65</v>
-      </c>
-      <c r="N57" t="s">
-        <v>65</v>
-      </c>
-      <c r="O57" t="s">
-        <v>65</v>
-      </c>
-      <c r="P57" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q57" t="s">
-        <v>65</v>
-      </c>
-      <c r="R57" t="s">
-        <v>64</v>
-      </c>
-      <c r="S57" t="s">
-        <v>65</v>
-      </c>
-      <c r="T57" t="s">
-        <v>65</v>
-      </c>
+      <c r="B57" s="5"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="5"/>
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="K57" s="5"/>
+      <c r="L57" s="5"/>
+      <c r="M57" s="5"/>
+      <c r="N57" s="5"/>
+      <c r="O57" s="5"/>
+      <c r="P57" s="5"/>
+      <c r="Q57" s="5"/>
+      <c r="R57" s="5"/>
+      <c r="S57" s="5"/>
+      <c r="T57" s="5"/>
     </row>
     <row r="58" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>42</v>
+        <v>76</v>
       </c>
       <c r="B58" t="s">
         <v>65</v>
@@ -3832,7 +3847,7 @@
     </row>
     <row r="59" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B59" t="s">
         <v>65</v>
@@ -3893,94 +3908,94 @@
       </c>
     </row>
     <row r="60" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B60" t="s">
+        <v>65</v>
+      </c>
+      <c r="C60" t="s">
+        <v>65</v>
+      </c>
+      <c r="D60" t="s">
+        <v>65</v>
+      </c>
+      <c r="E60" t="s">
+        <v>65</v>
+      </c>
+      <c r="F60" t="s">
+        <v>65</v>
+      </c>
+      <c r="G60" t="s">
+        <v>69</v>
+      </c>
+      <c r="H60" t="s">
+        <v>65</v>
+      </c>
+      <c r="I60" t="s">
+        <v>64</v>
+      </c>
+      <c r="J60" t="s">
+        <v>65</v>
+      </c>
+      <c r="K60" t="s">
+        <v>65</v>
+      </c>
+      <c r="L60" t="s">
+        <v>65</v>
+      </c>
+      <c r="M60" t="s">
+        <v>65</v>
+      </c>
+      <c r="N60" t="s">
+        <v>65</v>
+      </c>
+      <c r="O60" t="s">
+        <v>65</v>
+      </c>
+      <c r="P60" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q60" t="s">
+        <v>65</v>
+      </c>
+      <c r="R60" t="s">
+        <v>64</v>
+      </c>
+      <c r="S60" t="s">
+        <v>65</v>
+      </c>
+      <c r="T60" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B60" s="5"/>
-      <c r="C60" s="5"/>
-      <c r="D60" s="5"/>
-      <c r="E60" s="5"/>
-      <c r="F60" s="5"/>
-      <c r="G60" s="5"/>
-      <c r="H60" s="5"/>
-      <c r="I60" s="5"/>
-      <c r="J60" s="5"/>
-      <c r="K60" s="5"/>
-      <c r="L60" s="5"/>
-      <c r="M60" s="5"/>
-      <c r="N60" s="5"/>
-      <c r="O60" s="5"/>
-      <c r="P60" s="5"/>
-      <c r="Q60" s="5"/>
-      <c r="R60" s="5"/>
-      <c r="S60" s="5"/>
-      <c r="T60" s="5"/>
-    </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A61" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B61" t="s">
-        <v>65</v>
-      </c>
-      <c r="C61" t="s">
-        <v>65</v>
-      </c>
-      <c r="D61" t="s">
-        <v>65</v>
-      </c>
-      <c r="E61" t="s">
-        <v>65</v>
-      </c>
-      <c r="F61" t="s">
-        <v>65</v>
-      </c>
-      <c r="G61" t="s">
-        <v>69</v>
-      </c>
-      <c r="H61" t="s">
-        <v>65</v>
-      </c>
-      <c r="I61" t="s">
-        <v>64</v>
-      </c>
-      <c r="J61" t="s">
-        <v>65</v>
-      </c>
-      <c r="K61" t="s">
-        <v>65</v>
-      </c>
-      <c r="L61" t="s">
-        <v>65</v>
-      </c>
-      <c r="M61" t="s">
-        <v>65</v>
-      </c>
-      <c r="N61" t="s">
-        <v>65</v>
-      </c>
-      <c r="O61" t="s">
-        <v>65</v>
-      </c>
-      <c r="P61" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q61" t="s">
-        <v>65</v>
-      </c>
-      <c r="R61" t="s">
-        <v>64</v>
-      </c>
-      <c r="S61" t="s">
-        <v>65</v>
-      </c>
-      <c r="T61" t="s">
-        <v>65</v>
-      </c>
+      <c r="B61" s="5"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="5"/>
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="K61" s="5"/>
+      <c r="L61" s="5"/>
+      <c r="M61" s="5"/>
+      <c r="N61" s="5"/>
+      <c r="O61" s="5"/>
+      <c r="P61" s="5"/>
+      <c r="Q61" s="5"/>
+      <c r="R61" s="5"/>
+      <c r="S61" s="5"/>
+      <c r="T61" s="5"/>
     </row>
     <row r="62" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="B62" t="s">
         <v>65</v>
@@ -4041,94 +4056,94 @@
       </c>
     </row>
     <row r="63" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B63" t="s">
+        <v>65</v>
+      </c>
+      <c r="C63" t="s">
+        <v>65</v>
+      </c>
+      <c r="D63" t="s">
+        <v>65</v>
+      </c>
+      <c r="E63" t="s">
+        <v>65</v>
+      </c>
+      <c r="F63" t="s">
+        <v>65</v>
+      </c>
+      <c r="G63" t="s">
+        <v>69</v>
+      </c>
+      <c r="H63" t="s">
+        <v>65</v>
+      </c>
+      <c r="I63" t="s">
+        <v>64</v>
+      </c>
+      <c r="J63" t="s">
+        <v>65</v>
+      </c>
+      <c r="K63" t="s">
+        <v>65</v>
+      </c>
+      <c r="L63" t="s">
+        <v>65</v>
+      </c>
+      <c r="M63" t="s">
+        <v>65</v>
+      </c>
+      <c r="N63" t="s">
+        <v>65</v>
+      </c>
+      <c r="O63" t="s">
+        <v>65</v>
+      </c>
+      <c r="P63" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q63" t="s">
+        <v>65</v>
+      </c>
+      <c r="R63" t="s">
+        <v>64</v>
+      </c>
+      <c r="S63" t="s">
+        <v>65</v>
+      </c>
+      <c r="T63" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B63" s="5"/>
-      <c r="C63" s="5"/>
-      <c r="D63" s="5"/>
-      <c r="E63" s="5"/>
-      <c r="F63" s="5"/>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-      <c r="K63" s="5"/>
-      <c r="L63" s="5"/>
-      <c r="M63" s="5"/>
-      <c r="N63" s="5"/>
-      <c r="O63" s="5"/>
-      <c r="P63" s="5"/>
-      <c r="Q63" s="5"/>
-      <c r="R63" s="5"/>
-      <c r="S63" s="5"/>
-      <c r="T63" s="5"/>
-    </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A64" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B64" t="s">
-        <v>65</v>
-      </c>
-      <c r="C64" t="s">
-        <v>65</v>
-      </c>
-      <c r="D64" t="s">
-        <v>65</v>
-      </c>
-      <c r="E64" t="s">
-        <v>65</v>
-      </c>
-      <c r="F64" t="s">
-        <v>65</v>
-      </c>
-      <c r="G64" t="s">
-        <v>65</v>
-      </c>
-      <c r="H64" t="s">
-        <v>64</v>
-      </c>
-      <c r="I64" t="s">
-        <v>64</v>
-      </c>
-      <c r="J64" t="s">
-        <v>64</v>
-      </c>
-      <c r="K64" t="s">
-        <v>65</v>
-      </c>
-      <c r="L64" t="s">
-        <v>65</v>
-      </c>
-      <c r="M64" t="s">
-        <v>65</v>
-      </c>
-      <c r="N64" t="s">
-        <v>70</v>
-      </c>
-      <c r="O64" t="s">
-        <v>65</v>
-      </c>
-      <c r="P64" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q64" t="s">
-        <v>65</v>
-      </c>
-      <c r="R64" t="s">
-        <v>68</v>
-      </c>
-      <c r="S64" t="s">
-        <v>65</v>
-      </c>
-      <c r="T64" t="s">
-        <v>65</v>
-      </c>
+      <c r="B64" s="5"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="5"/>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="5"/>
+      <c r="K64" s="5"/>
+      <c r="L64" s="5"/>
+      <c r="M64" s="5"/>
+      <c r="N64" s="5"/>
+      <c r="O64" s="5"/>
+      <c r="P64" s="5"/>
+      <c r="Q64" s="5"/>
+      <c r="R64" s="5"/>
+      <c r="S64" s="5"/>
+      <c r="T64" s="5"/>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="B65" t="s">
         <v>65</v>
@@ -4190,7 +4205,7 @@
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B66" t="s">
         <v>65</v>
@@ -4214,10 +4229,10 @@
         <v>64</v>
       </c>
       <c r="I66" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="J66" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="K66" t="s">
         <v>65</v>
@@ -4251,94 +4266,94 @@
       </c>
     </row>
     <row r="67" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A67" s="5" t="s">
+      <c r="A67" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B67" t="s">
+        <v>65</v>
+      </c>
+      <c r="C67" t="s">
+        <v>65</v>
+      </c>
+      <c r="D67" t="s">
+        <v>65</v>
+      </c>
+      <c r="E67" t="s">
+        <v>65</v>
+      </c>
+      <c r="F67" t="s">
+        <v>65</v>
+      </c>
+      <c r="G67" t="s">
+        <v>65</v>
+      </c>
+      <c r="H67" t="s">
+        <v>64</v>
+      </c>
+      <c r="I67" t="s">
+        <v>66</v>
+      </c>
+      <c r="J67" t="s">
+        <v>66</v>
+      </c>
+      <c r="K67" t="s">
+        <v>65</v>
+      </c>
+      <c r="L67" t="s">
+        <v>65</v>
+      </c>
+      <c r="M67" t="s">
+        <v>65</v>
+      </c>
+      <c r="N67" t="s">
+        <v>70</v>
+      </c>
+      <c r="O67" t="s">
+        <v>65</v>
+      </c>
+      <c r="P67" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q67" t="s">
+        <v>65</v>
+      </c>
+      <c r="R67" t="s">
+        <v>68</v>
+      </c>
+      <c r="S67" t="s">
+        <v>65</v>
+      </c>
+      <c r="T67" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A68" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B67" s="5"/>
-      <c r="C67" s="5"/>
-      <c r="D67" s="5"/>
-      <c r="E67" s="5"/>
-      <c r="F67" s="5"/>
-      <c r="G67" s="5"/>
-      <c r="H67" s="5"/>
-      <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
-      <c r="K67" s="5"/>
-      <c r="L67" s="5"/>
-      <c r="M67" s="5"/>
-      <c r="N67" s="5"/>
-      <c r="O67" s="5"/>
-      <c r="P67" s="5"/>
-      <c r="Q67" s="5"/>
-      <c r="R67" s="5"/>
-      <c r="S67" s="5"/>
-      <c r="T67" s="5"/>
-    </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
-      <c r="A68" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="B68" t="s">
-        <v>65</v>
-      </c>
-      <c r="C68" t="s">
-        <v>65</v>
-      </c>
-      <c r="D68" t="s">
-        <v>65</v>
-      </c>
-      <c r="E68" t="s">
-        <v>65</v>
-      </c>
-      <c r="F68" t="s">
-        <v>65</v>
-      </c>
-      <c r="G68" t="s">
-        <v>65</v>
-      </c>
-      <c r="H68" t="s">
-        <v>64</v>
-      </c>
-      <c r="I68" t="s">
-        <v>64</v>
-      </c>
-      <c r="J68" t="s">
-        <v>64</v>
-      </c>
-      <c r="K68" t="s">
-        <v>65</v>
-      </c>
-      <c r="L68" t="s">
-        <v>65</v>
-      </c>
-      <c r="M68" t="s">
-        <v>65</v>
-      </c>
-      <c r="N68" t="s">
-        <v>70</v>
-      </c>
-      <c r="O68" t="s">
-        <v>65</v>
-      </c>
-      <c r="P68" t="s">
-        <v>70</v>
-      </c>
-      <c r="Q68" t="s">
-        <v>65</v>
-      </c>
-      <c r="R68" t="s">
-        <v>64</v>
-      </c>
-      <c r="S68" t="s">
-        <v>65</v>
-      </c>
-      <c r="T68" t="s">
-        <v>69</v>
-      </c>
+      <c r="B68" s="5"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="5"/>
+      <c r="G68" s="5"/>
+      <c r="H68" s="5"/>
+      <c r="I68" s="5"/>
+      <c r="J68" s="5"/>
+      <c r="K68" s="5"/>
+      <c r="L68" s="5"/>
+      <c r="M68" s="5"/>
+      <c r="N68" s="5"/>
+      <c r="O68" s="5"/>
+      <c r="P68" s="5"/>
+      <c r="Q68" s="5"/>
+      <c r="R68" s="5"/>
+      <c r="S68" s="5"/>
+      <c r="T68" s="5"/>
     </row>
     <row r="69" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B69" t="s">
         <v>65</v>
@@ -4383,7 +4398,7 @@
         <v>65</v>
       </c>
       <c r="P69" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="Q69" t="s">
         <v>65</v>
@@ -4396,6 +4411,364 @@
       </c>
       <c r="T69" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B70" t="s">
+        <v>65</v>
+      </c>
+      <c r="C70" t="s">
+        <v>65</v>
+      </c>
+      <c r="D70" t="s">
+        <v>65</v>
+      </c>
+      <c r="E70" t="s">
+        <v>65</v>
+      </c>
+      <c r="F70" t="s">
+        <v>65</v>
+      </c>
+      <c r="G70" t="s">
+        <v>65</v>
+      </c>
+      <c r="H70" t="s">
+        <v>64</v>
+      </c>
+      <c r="I70" t="s">
+        <v>64</v>
+      </c>
+      <c r="J70" t="s">
+        <v>64</v>
+      </c>
+      <c r="K70" t="s">
+        <v>65</v>
+      </c>
+      <c r="L70" t="s">
+        <v>65</v>
+      </c>
+      <c r="M70" t="s">
+        <v>65</v>
+      </c>
+      <c r="N70" t="s">
+        <v>70</v>
+      </c>
+      <c r="O70" t="s">
+        <v>65</v>
+      </c>
+      <c r="P70" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q70" t="s">
+        <v>65</v>
+      </c>
+      <c r="R70" t="s">
+        <v>64</v>
+      </c>
+      <c r="S70" t="s">
+        <v>65</v>
+      </c>
+      <c r="T70" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="B71" s="5"/>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="5"/>
+      <c r="G71" s="5"/>
+      <c r="H71" s="5"/>
+      <c r="I71" s="5"/>
+      <c r="J71" s="5"/>
+      <c r="K71" s="5"/>
+      <c r="L71" s="5"/>
+      <c r="M71" s="5"/>
+      <c r="N71" s="5"/>
+      <c r="O71" s="5"/>
+      <c r="P71" s="5"/>
+      <c r="Q71" s="5"/>
+      <c r="R71" s="5"/>
+      <c r="S71" s="5"/>
+      <c r="T71" s="5"/>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B72" t="s">
+        <v>65</v>
+      </c>
+      <c r="C72" t="s">
+        <v>65</v>
+      </c>
+      <c r="D72" t="s">
+        <v>65</v>
+      </c>
+      <c r="E72" t="s">
+        <v>65</v>
+      </c>
+      <c r="F72" t="s">
+        <v>65</v>
+      </c>
+      <c r="G72" t="s">
+        <v>65</v>
+      </c>
+      <c r="H72" t="s">
+        <v>64</v>
+      </c>
+      <c r="I72" t="s">
+        <v>65</v>
+      </c>
+      <c r="J72" t="s">
+        <v>65</v>
+      </c>
+      <c r="K72" t="s">
+        <v>65</v>
+      </c>
+      <c r="L72" t="s">
+        <v>65</v>
+      </c>
+      <c r="M72" t="s">
+        <v>65</v>
+      </c>
+      <c r="N72" t="s">
+        <v>65</v>
+      </c>
+      <c r="O72" t="s">
+        <v>65</v>
+      </c>
+      <c r="P72" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q72" t="s">
+        <v>65</v>
+      </c>
+      <c r="R72" t="s">
+        <v>64</v>
+      </c>
+      <c r="S72" t="s">
+        <v>65</v>
+      </c>
+      <c r="T72" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B73" t="s">
+        <v>65</v>
+      </c>
+      <c r="C73" t="s">
+        <v>65</v>
+      </c>
+      <c r="D73" t="s">
+        <v>65</v>
+      </c>
+      <c r="E73" t="s">
+        <v>65</v>
+      </c>
+      <c r="F73" t="s">
+        <v>65</v>
+      </c>
+      <c r="G73" t="s">
+        <v>65</v>
+      </c>
+      <c r="H73" t="s">
+        <v>65</v>
+      </c>
+      <c r="I73" t="s">
+        <v>65</v>
+      </c>
+      <c r="J73" t="s">
+        <v>65</v>
+      </c>
+      <c r="K73" t="s">
+        <v>65</v>
+      </c>
+      <c r="L73" t="s">
+        <v>65</v>
+      </c>
+      <c r="M73" t="s">
+        <v>65</v>
+      </c>
+      <c r="N73" t="s">
+        <v>65</v>
+      </c>
+      <c r="O73" t="s">
+        <v>65</v>
+      </c>
+      <c r="P73" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q73" t="s">
+        <v>65</v>
+      </c>
+      <c r="R73" t="s">
+        <v>64</v>
+      </c>
+      <c r="S73" t="s">
+        <v>65</v>
+      </c>
+      <c r="T73" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A74" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B74" s="5"/>
+      <c r="C74" s="5"/>
+      <c r="D74" s="5"/>
+      <c r="E74" s="5"/>
+      <c r="F74" s="5"/>
+      <c r="G74" s="5"/>
+      <c r="H74" s="5"/>
+      <c r="I74" s="5"/>
+      <c r="J74" s="5"/>
+      <c r="K74" s="5"/>
+      <c r="L74" s="5"/>
+      <c r="M74" s="5"/>
+      <c r="N74" s="5"/>
+      <c r="O74" s="5"/>
+      <c r="P74" s="5"/>
+      <c r="Q74" s="5"/>
+      <c r="R74" s="5"/>
+      <c r="S74" s="5"/>
+      <c r="T74" s="5"/>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A75" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B75" t="s">
+        <v>65</v>
+      </c>
+      <c r="C75" t="s">
+        <v>65</v>
+      </c>
+      <c r="D75" t="s">
+        <v>65</v>
+      </c>
+      <c r="E75" t="s">
+        <v>65</v>
+      </c>
+      <c r="F75" t="s">
+        <v>65</v>
+      </c>
+      <c r="G75" t="s">
+        <v>65</v>
+      </c>
+      <c r="H75" t="s">
+        <v>64</v>
+      </c>
+      <c r="I75" t="s">
+        <v>65</v>
+      </c>
+      <c r="J75" t="s">
+        <v>65</v>
+      </c>
+      <c r="K75" t="s">
+        <v>65</v>
+      </c>
+      <c r="L75" t="s">
+        <v>65</v>
+      </c>
+      <c r="M75" t="s">
+        <v>65</v>
+      </c>
+      <c r="N75" t="s">
+        <v>65</v>
+      </c>
+      <c r="O75" t="s">
+        <v>65</v>
+      </c>
+      <c r="P75" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q75" t="s">
+        <v>65</v>
+      </c>
+      <c r="R75" t="s">
+        <v>64</v>
+      </c>
+      <c r="S75" t="s">
+        <v>65</v>
+      </c>
+      <c r="T75" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B76" t="s">
+        <v>65</v>
+      </c>
+      <c r="C76" t="s">
+        <v>65</v>
+      </c>
+      <c r="D76" t="s">
+        <v>65</v>
+      </c>
+      <c r="E76" t="s">
+        <v>65</v>
+      </c>
+      <c r="F76" t="s">
+        <v>65</v>
+      </c>
+      <c r="G76" t="s">
+        <v>65</v>
+      </c>
+      <c r="H76" t="s">
+        <v>64</v>
+      </c>
+      <c r="I76" t="s">
+        <v>65</v>
+      </c>
+      <c r="J76" t="s">
+        <v>65</v>
+      </c>
+      <c r="K76" t="s">
+        <v>65</v>
+      </c>
+      <c r="L76" t="s">
+        <v>65</v>
+      </c>
+      <c r="M76" t="s">
+        <v>65</v>
+      </c>
+      <c r="N76" t="s">
+        <v>65</v>
+      </c>
+      <c r="O76" t="s">
+        <v>65</v>
+      </c>
+      <c r="P76" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q76" t="s">
+        <v>65</v>
+      </c>
+      <c r="R76" t="s">
+        <v>64</v>
+      </c>
+      <c r="S76" t="s">
+        <v>65</v>
+      </c>
+      <c r="T76" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>